<commit_message>
Add configurable character cards
</commit_message>
<xml_diff>
--- a/external/config/cards.xlsx
+++ b/external/config/cards.xlsx
@@ -349,7 +349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BX68"/>
+  <dimension ref="A1:CD83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -782,6 +782,36 @@
           <t>upgrade_pickable_cards_max_amount</t>
         </is>
       </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>card_values_json</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>card_play_actions_json</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>card_draw_actions_json</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>card_discard_actions_json</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>card_retain_actions_json</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>card_listeners_json</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6491,6 +6521,1660 @@
       <c r="AU68" t="n">
         <v>0</v>
       </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>card_hasty_sorting</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>慌忙整理</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>弃置最多 [max_card_amount] 张牌。每弃置1张，抽 [draw_count] 张牌。</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J69" t="b">
+        <v>0</v>
+      </c>
+      <c r="K69" t="b">
+        <v>0</v>
+      </c>
+      <c r="L69" t="b">
+        <v>0</v>
+      </c>
+      <c r="M69" t="b">
+        <v>0</v>
+      </c>
+      <c r="N69" t="b">
+        <v>1</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/blue/card_blue.png</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>keyword_discard</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="n">
+        <v>1</v>
+      </c>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="inlineStr"/>
+      <c r="W69" t="inlineStr"/>
+      <c r="X69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr"/>
+      <c r="Z69" t="inlineStr"/>
+      <c r="AA69" t="inlineStr"/>
+      <c r="AB69" t="inlineStr"/>
+      <c r="AC69" t="inlineStr"/>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE69" t="inlineStr"/>
+      <c r="AK69" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW69" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX69" t="inlineStr"/>
+      <c r="BW69" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY69" t="inlineStr">
+        <is>
+          <t>{"draw_count":1,"min_card_amount":0,"max_card_amount":2}</t>
+        </is>
+      </c>
+      <c r="BZ69" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":0,"max_card_amount":2,"card_pick_type":0,"card_pick_text":"选择最多 {0} 张牌弃掉。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionDiscardCards.gd":{}},{"res://scripts/actions/meta_actions/ActionVariableCardsetModifier.gd":{"multiplied_values":["draw_count"],"action_data":[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"draw_count":1}}]}}],"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA69" t="inlineStr"/>
+      <c r="CB69" t="inlineStr"/>
+      <c r="CC69" t="inlineStr"/>
+      <c r="CD69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>card_something_fell_out</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>掉出来了</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>无法打出。被手动弃置时获得 [energy_amount] 点能量。</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J70" t="b">
+        <v>0</v>
+      </c>
+      <c r="K70" t="b">
+        <v>0</v>
+      </c>
+      <c r="L70" t="b">
+        <v>0</v>
+      </c>
+      <c r="M70" t="b">
+        <v>0</v>
+      </c>
+      <c r="N70" t="b">
+        <v>1</v>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/blue/card_blue.png</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>keyword_discard</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="inlineStr"/>
+      <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr"/>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr"/>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr"/>
+      <c r="AK70" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV70" t="inlineStr"/>
+      <c r="AW70" t="inlineStr"/>
+      <c r="AX70" t="inlineStr"/>
+      <c r="BY70" t="inlineStr">
+        <is>
+          <t>{"energy_amount":2}</t>
+        </is>
+      </c>
+      <c r="BZ70" t="inlineStr"/>
+      <c r="CA70" t="inlineStr"/>
+      <c r="CB70" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/ActionAddEnergy.gd":{"energy_amount":2,"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CC70" t="inlineStr"/>
+      <c r="CD70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>card_quick_search</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>临时翻找</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>从弃牌堆选择 [max_card_amount] 张牌加入手牌。本回合其费用变为0。</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J71" t="b">
+        <v>0</v>
+      </c>
+      <c r="K71" t="b">
+        <v>0</v>
+      </c>
+      <c r="L71" t="b">
+        <v>0</v>
+      </c>
+      <c r="M71" t="b">
+        <v>0</v>
+      </c>
+      <c r="N71" t="b">
+        <v>1</v>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/blue/card_blue.png</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="inlineStr"/>
+      <c r="W71" t="inlineStr"/>
+      <c r="X71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr"/>
+      <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr"/>
+      <c r="AB71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr"/>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr"/>
+      <c r="AK71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX71" t="inlineStr"/>
+      <c r="BY71" t="inlineStr">
+        <is>
+          <t>{"min_card_amount":1,"max_card_amount":1}</t>
+        </is>
+      </c>
+      <c r="BZ71" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"card_pick_type":4,"card_pick_text":"从弃牌堆选择 {0} 张牌。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionAddCardsToHand.gd":{}},{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd":{"card_energy_cost_until_turn":0}}],"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA71" t="inlineStr"/>
+      <c r="CB71" t="inlineStr"/>
+      <c r="CC71" t="inlineStr"/>
+      <c r="CD71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>card_by_accident</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>误打误撞</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>随机打出弃牌堆中的 [max_card_amount] 张牌。</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J72" t="b">
+        <v>0</v>
+      </c>
+      <c r="K72" t="b">
+        <v>0</v>
+      </c>
+      <c r="L72" t="b">
+        <v>0</v>
+      </c>
+      <c r="M72" t="b">
+        <v>0</v>
+      </c>
+      <c r="N72" t="b">
+        <v>1</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/blue/card_blue.png</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
+      <c r="V72" t="inlineStr"/>
+      <c r="W72" t="inlineStr"/>
+      <c r="X72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr"/>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="inlineStr"/>
+      <c r="AC72" t="inlineStr"/>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE72" t="inlineStr"/>
+      <c r="AK72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX72" t="inlineStr"/>
+      <c r="BY72" t="inlineStr">
+        <is>
+          <t>{"min_card_amount":1,"max_card_amount":1}</t>
+        </is>
+      </c>
+      <c r="BZ72" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"random_selection":true,"card_pick_type":4,"action_data":[{"res://scripts/actions/cardset_actions/ActionPlayCards.gd":{}}],"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA72" t="inlineStr"/>
+      <c r="CB72" t="inlineStr"/>
+      <c r="CC72" t="inlineStr"/>
+      <c r="CD72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>card_backup_drink</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>备用饮料</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>生成一个随机消耗品。如果本回合弃置过牌，抽 [draw_count] 张牌。放逐。</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>color_blue</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J73" t="b">
+        <v>0</v>
+      </c>
+      <c r="K73" t="b">
+        <v>1</v>
+      </c>
+      <c r="L73" t="b">
+        <v>0</v>
+      </c>
+      <c r="M73" t="b">
+        <v>0</v>
+      </c>
+      <c r="N73" t="b">
+        <v>1</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/blue/card_blue.png</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="n">
+        <v>1</v>
+      </c>
+      <c r="U73" t="inlineStr"/>
+      <c r="V73" t="inlineStr"/>
+      <c r="W73" t="inlineStr"/>
+      <c r="X73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr"/>
+      <c r="Z73" t="inlineStr"/>
+      <c r="AA73" t="inlineStr"/>
+      <c r="AB73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr"/>
+      <c r="AK73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV73" t="inlineStr"/>
+      <c r="AW73" t="inlineStr"/>
+      <c r="AX73" t="inlineStr"/>
+      <c r="BY73" t="inlineStr">
+        <is>
+          <t>{"draw_count":1,"random_consumable":1,"fill_all_slots":0}</t>
+        </is>
+      </c>
+      <c r="BZ73" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/player_actions/ActionAddConsumable.gd":{"random_consumable":1,"fill_all_slots":0,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/ValidatorCombatStats.gd":{"stat_enum":13,"is_total_stat":false,"operator":"&gt;","comparison_value":0}}],"passed_action_data":[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA73" t="inlineStr"/>
+      <c r="CB73" t="inlineStr"/>
+      <c r="CC73" t="inlineStr"/>
+      <c r="CD73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>card_first_beat</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>第一拍</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>获得 [block] 点格挡。如果这是本回合打出的第一张牌，额外抽 [draw_count] 张牌。</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J74" t="b">
+        <v>0</v>
+      </c>
+      <c r="K74" t="b">
+        <v>0</v>
+      </c>
+      <c r="L74" t="b">
+        <v>0</v>
+      </c>
+      <c r="M74" t="b">
+        <v>0</v>
+      </c>
+      <c r="N74" t="b">
+        <v>1</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>keyword_block</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="n">
+        <v>6</v>
+      </c>
+      <c r="T74" t="n">
+        <v>1</v>
+      </c>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="inlineStr"/>
+      <c r="W74" t="inlineStr"/>
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr"/>
+      <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr"/>
+      <c r="AB74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr"/>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr"/>
+      <c r="AK74" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN74" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV74" t="inlineStr"/>
+      <c r="AW74" t="inlineStr"/>
+      <c r="AX74" t="inlineStr"/>
+      <c r="BY74" t="inlineStr">
+        <is>
+          <t>{"block":6,"draw_count":1}</t>
+        </is>
+      </c>
+      <c r="BZ74" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/ActionBlock.gd":{"time_delay":0.5,"target_override":1,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/ValidatorCombatStats.gd":{"stat_enum":11,"is_total_stat":false,"operator":"==","comparison_value":0}}],"passed_action_data":[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"draw_count":1}}],"failed_action_data":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA74" t="inlineStr"/>
+      <c r="CB74" t="inlineStr"/>
+      <c r="CC74" t="inlineStr"/>
+      <c r="CD74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>card_distorted_note</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>失真音</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>造成 [damage] 点伤害并施加 [status_charge_amount] 层腐蚀。如果目标正在攻击，切换其意图。</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J75" t="b">
+        <v>1</v>
+      </c>
+      <c r="K75" t="b">
+        <v>0</v>
+      </c>
+      <c r="L75" t="b">
+        <v>0</v>
+      </c>
+      <c r="M75" t="b">
+        <v>0</v>
+      </c>
+      <c r="N75" t="b">
+        <v>1</v>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>keyword_corrosion</t>
+        </is>
+      </c>
+      <c r="Q75" t="n">
+        <v>5</v>
+      </c>
+      <c r="R75" t="n">
+        <v>1</v>
+      </c>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="n">
+        <v>4</v>
+      </c>
+      <c r="V75" t="inlineStr"/>
+      <c r="W75" t="inlineStr"/>
+      <c r="X75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr"/>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>status_effect_corrosion</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr"/>
+      <c r="AB75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr"/>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr"/>
+      <c r="AK75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM75" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ75" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV75" t="inlineStr"/>
+      <c r="AW75" t="inlineStr"/>
+      <c r="AX75" t="inlineStr"/>
+      <c r="BY75" t="inlineStr">
+        <is>
+          <t>{"damage":5,"number_of_attacks":1,"status_charge_amount":4,"status_effect_object_id":"status_effect_corrosion"}</t>
+        </is>
+      </c>
+      <c r="BZ75" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"time_delay":0.0,"actions_on_lethal":[]}},{"res://scripts/actions/status_actions/ActionApplyStatus.gd":{"time_delay":0.5,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd":{}}],"passed_action_data":[{"res://scripts/actions/enemy_actions/ActionCycleEnemyIntent.gd":{"time_delay":0.0,"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA75" t="inlineStr"/>
+      <c r="CB75" t="inlineStr"/>
+      <c r="CC75" t="inlineStr"/>
+      <c r="CD75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>card_tuning</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>调音</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>选择1张手牌。本场战斗中其伤害和格挡提高 [improve_amount]。放逐。</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+      <c r="K76" t="b">
+        <v>1</v>
+      </c>
+      <c r="L76" t="b">
+        <v>0</v>
+      </c>
+      <c r="M76" t="b">
+        <v>0</v>
+      </c>
+      <c r="N76" t="b">
+        <v>1</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
+      <c r="U76" t="inlineStr"/>
+      <c r="V76" t="inlineStr"/>
+      <c r="W76" t="inlineStr"/>
+      <c r="X76" t="inlineStr"/>
+      <c r="Y76" t="inlineStr"/>
+      <c r="Z76" t="inlineStr"/>
+      <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
+      <c r="AC76" t="inlineStr"/>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr"/>
+      <c r="AK76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX76" t="inlineStr"/>
+      <c r="BY76" t="inlineStr">
+        <is>
+          <t>{"improve_amount":2,"min_card_amount":1,"max_card_amount":1}</t>
+        </is>
+      </c>
+      <c r="BZ76" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"card_pick_type":0,"card_pick_text":"选择 {0} 张牌调音。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd":{"improve_parent_card":false,"card_value_improvements":{"damage":2,"block":2}}}],"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA76" t="inlineStr"/>
+      <c r="CB76" t="inlineStr"/>
+      <c r="CC76" t="inlineStr"/>
+      <c r="CD76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>card_warmup</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>赛前热身</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>保留。获得 [block] 点格挡。每次被保留时，格挡提高 [improve_amount]。</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J77" t="b">
+        <v>0</v>
+      </c>
+      <c r="K77" t="b">
+        <v>0</v>
+      </c>
+      <c r="L77" t="b">
+        <v>0</v>
+      </c>
+      <c r="M77" t="b">
+        <v>1</v>
+      </c>
+      <c r="N77" t="b">
+        <v>1</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>keyword_block,keyword_retain</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="n">
+        <v>6</v>
+      </c>
+      <c r="T77" t="inlineStr"/>
+      <c r="U77" t="inlineStr"/>
+      <c r="V77" t="inlineStr"/>
+      <c r="W77" t="inlineStr"/>
+      <c r="X77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr"/>
+      <c r="Z77" t="inlineStr"/>
+      <c r="AA77" t="inlineStr"/>
+      <c r="AB77" t="inlineStr"/>
+      <c r="AC77" t="inlineStr"/>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE77" t="inlineStr"/>
+      <c r="AK77" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN77" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV77" t="inlineStr"/>
+      <c r="AW77" t="inlineStr"/>
+      <c r="AX77" t="inlineStr"/>
+      <c r="BY77" t="inlineStr">
+        <is>
+          <t>{"block":6,"improve_amount":2}</t>
+        </is>
+      </c>
+      <c r="BZ77" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/ActionBlock.gd":{"time_delay":0.5,"target_override":1,"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA77" t="inlineStr"/>
+      <c r="CB77" t="inlineStr"/>
+      <c r="CC77" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd":{"pick_played_card":true,"improve_parent_card":false,"card_value_improvements":{"block":2}}}]</t>
+        </is>
+      </c>
+      <c r="CD77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>card_sports_drink</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>运动饮料</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>抽到时获得 [energy_amount] 点能量。打出时抽 [draw_count] 张牌。放逐。</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J78" t="b">
+        <v>0</v>
+      </c>
+      <c r="K78" t="b">
+        <v>1</v>
+      </c>
+      <c r="L78" t="b">
+        <v>0</v>
+      </c>
+      <c r="M78" t="b">
+        <v>0</v>
+      </c>
+      <c r="N78" t="b">
+        <v>1</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>keyword_exhaust</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="n">
+        <v>1</v>
+      </c>
+      <c r="U78" t="inlineStr"/>
+      <c r="V78" t="inlineStr"/>
+      <c r="W78" t="inlineStr"/>
+      <c r="X78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr"/>
+      <c r="Z78" t="inlineStr"/>
+      <c r="AA78" t="inlineStr"/>
+      <c r="AB78" t="inlineStr"/>
+      <c r="AC78" t="inlineStr"/>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr"/>
+      <c r="AK78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV78" t="inlineStr"/>
+      <c r="AW78" t="inlineStr"/>
+      <c r="AX78" t="inlineStr"/>
+      <c r="BY78" t="inlineStr">
+        <is>
+          <t>{"energy_amount":1,"draw_count":1}</t>
+        </is>
+      </c>
+      <c r="BZ78" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA78" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/ActionAddEnergy.gd":{"energy_amount":1,"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CB78" t="inlineStr"/>
+      <c r="CC78" t="inlineStr"/>
+      <c r="CD78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>card_bag_swing</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>甩包冲撞</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>造成 [damage] 点伤害。如果本回合有牌被放逐，额外造成 [bonus_damage] 点伤害。</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J79" t="b">
+        <v>1</v>
+      </c>
+      <c r="K79" t="b">
+        <v>0</v>
+      </c>
+      <c r="L79" t="b">
+        <v>0</v>
+      </c>
+      <c r="M79" t="b">
+        <v>0</v>
+      </c>
+      <c r="N79" t="b">
+        <v>1</v>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="n">
+        <v>7</v>
+      </c>
+      <c r="R79" t="n">
+        <v>1</v>
+      </c>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
+      <c r="U79" t="inlineStr"/>
+      <c r="V79" t="inlineStr"/>
+      <c r="W79" t="inlineStr"/>
+      <c r="X79" t="inlineStr"/>
+      <c r="Y79" t="inlineStr"/>
+      <c r="Z79" t="inlineStr"/>
+      <c r="AA79" t="inlineStr"/>
+      <c r="AB79" t="inlineStr"/>
+      <c r="AC79" t="inlineStr"/>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr"/>
+      <c r="AK79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM79" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV79" t="inlineStr"/>
+      <c r="AW79" t="inlineStr"/>
+      <c r="AX79" t="inlineStr"/>
+      <c r="BY79" t="inlineStr">
+        <is>
+          <t>{"damage":7,"bonus_damage":8,"number_of_attacks":1}</t>
+        </is>
+      </c>
+      <c r="BZ79" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"time_delay":0.0,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/ValidatorCombatStats.gd":{"stat_enum":14,"is_total_stat":false,"operator":"&gt;","comparison_value":0}}],"passed_action_data":[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"custom_key_names":{"damage":"bonus_damage"},"number_of_attacks":1,"time_delay":0.0,"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA79" t="inlineStr"/>
+      <c r="CB79" t="inlineStr"/>
+      <c r="CC79" t="inlineStr"/>
+      <c r="CD79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>card_old_item_reuse</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>旧物回收</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>放逐1张手牌。获得 [block] 点格挡，抽 [draw_count] 张牌。</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J80" t="b">
+        <v>0</v>
+      </c>
+      <c r="K80" t="b">
+        <v>0</v>
+      </c>
+      <c r="L80" t="b">
+        <v>0</v>
+      </c>
+      <c r="M80" t="b">
+        <v>0</v>
+      </c>
+      <c r="N80" t="b">
+        <v>1</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>keyword_exhaust,keyword_block</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="n">
+        <v>6</v>
+      </c>
+      <c r="T80" t="n">
+        <v>1</v>
+      </c>
+      <c r="U80" t="inlineStr"/>
+      <c r="V80" t="inlineStr"/>
+      <c r="W80" t="inlineStr"/>
+      <c r="X80" t="inlineStr"/>
+      <c r="Y80" t="inlineStr"/>
+      <c r="Z80" t="inlineStr"/>
+      <c r="AA80" t="inlineStr"/>
+      <c r="AB80" t="inlineStr"/>
+      <c r="AC80" t="inlineStr"/>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr"/>
+      <c r="AK80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN80" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX80" t="inlineStr"/>
+      <c r="BY80" t="inlineStr">
+        <is>
+          <t>{"block":6,"draw_count":1,"min_card_amount":1,"max_card_amount":1}</t>
+        </is>
+      </c>
+      <c r="BZ80" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"card_pick_type":0,"card_pick_text":"选择 {0} 张牌放逐。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionExhaustCards.gd":{}},{"res://scripts/actions/ActionBlock.gd":{"target_override":1,"time_delay":0.5}},{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"draw_count":1}}],"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA80" t="inlineStr"/>
+      <c r="CB80" t="inlineStr"/>
+      <c r="CC80" t="inlineStr"/>
+      <c r="CD80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>card_sprint_start</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>冲刺起跑</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>抽到时，本回合费用变为0。造成 [damage] 点伤害。</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J81" t="b">
+        <v>1</v>
+      </c>
+      <c r="K81" t="b">
+        <v>0</v>
+      </c>
+      <c r="L81" t="b">
+        <v>0</v>
+      </c>
+      <c r="M81" t="b">
+        <v>0</v>
+      </c>
+      <c r="N81" t="b">
+        <v>1</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="n">
+        <v>12</v>
+      </c>
+      <c r="R81" t="n">
+        <v>1</v>
+      </c>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
+      <c r="U81" t="inlineStr"/>
+      <c r="V81" t="inlineStr"/>
+      <c r="W81" t="inlineStr"/>
+      <c r="X81" t="inlineStr"/>
+      <c r="Y81" t="inlineStr"/>
+      <c r="Z81" t="inlineStr"/>
+      <c r="AA81" t="inlineStr"/>
+      <c r="AB81" t="inlineStr"/>
+      <c r="AC81" t="inlineStr"/>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE81" t="inlineStr"/>
+      <c r="AK81" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM81" t="n">
+        <v>4</v>
+      </c>
+      <c r="AU81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV81" t="inlineStr"/>
+      <c r="AW81" t="inlineStr"/>
+      <c r="AX81" t="inlineStr"/>
+      <c r="BY81" t="inlineStr">
+        <is>
+          <t>{"damage":12,"number_of_attacks":1}</t>
+        </is>
+      </c>
+      <c r="BZ81" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"time_delay":0.0,"actions_on_lethal":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA81" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd":{"pick_played_card":true,"card_energy_cost_until_turn":0}}]</t>
+        </is>
+      </c>
+      <c r="CB81" t="inlineStr"/>
+      <c r="CC81" t="inlineStr"/>
+      <c r="CD81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>card_opening_strike</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>破绽打击</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>造成 [damage] 点伤害。如果目标正在攻击，施加 [status_charge_amount] 层易伤。</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>color_red</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J82" t="b">
+        <v>1</v>
+      </c>
+      <c r="K82" t="b">
+        <v>0</v>
+      </c>
+      <c r="L82" t="b">
+        <v>0</v>
+      </c>
+      <c r="M82" t="b">
+        <v>0</v>
+      </c>
+      <c r="N82" t="b">
+        <v>1</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/red/card_red.png</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="n">
+        <v>7</v>
+      </c>
+      <c r="R82" t="n">
+        <v>1</v>
+      </c>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr"/>
+      <c r="U82" t="n">
+        <v>2</v>
+      </c>
+      <c r="V82" t="inlineStr"/>
+      <c r="W82" t="inlineStr"/>
+      <c r="X82" t="inlineStr"/>
+      <c r="Y82" t="inlineStr"/>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>status_effect_vulnerable</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr"/>
+      <c r="AB82" t="inlineStr"/>
+      <c r="AC82" t="inlineStr"/>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE82" t="inlineStr"/>
+      <c r="AK82" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM82" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV82" t="inlineStr"/>
+      <c r="AW82" t="inlineStr"/>
+      <c r="AX82" t="inlineStr"/>
+      <c r="BY82" t="inlineStr">
+        <is>
+          <t>{"damage":7,"number_of_attacks":1,"status_charge_amount":2,"status_effect_object_id":"status_effect_vulnerable"}</t>
+        </is>
+      </c>
+      <c r="BZ82" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"time_delay":0.0,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd":{}}],"passed_action_data":[{"res://scripts/actions/status_actions/ActionApplyStatus.gd":{"status_charge_amount":2,"status_effect_object_id":"status_effect_vulnerable","time_delay":0.5,"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
+        </is>
+      </c>
+      <c r="CA82" t="inlineStr"/>
+      <c r="CB82" t="inlineStr"/>
+      <c r="CC82" t="inlineStr"/>
+      <c r="CD82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>card_finisher</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>终结拳</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>造成 [damage] 点伤害。本回合每打出过1张牌，额外造成 [damage_per_card] 点伤害。</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>3</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>color_red</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>2</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J83" t="b">
+        <v>1</v>
+      </c>
+      <c r="K83" t="b">
+        <v>0</v>
+      </c>
+      <c r="L83" t="b">
+        <v>0</v>
+      </c>
+      <c r="M83" t="b">
+        <v>0</v>
+      </c>
+      <c r="N83" t="b">
+        <v>1</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/red/card_red.png</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="n">
+        <v>12</v>
+      </c>
+      <c r="R83" t="n">
+        <v>1</v>
+      </c>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr"/>
+      <c r="U83" t="inlineStr"/>
+      <c r="V83" t="inlineStr"/>
+      <c r="W83" t="inlineStr"/>
+      <c r="X83" t="inlineStr"/>
+      <c r="Y83" t="inlineStr"/>
+      <c r="Z83" t="inlineStr"/>
+      <c r="AA83" t="inlineStr"/>
+      <c r="AB83" t="inlineStr"/>
+      <c r="AC83" t="inlineStr"/>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="AE83" t="inlineStr"/>
+      <c r="AK83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV83" t="inlineStr"/>
+      <c r="AW83" t="inlineStr"/>
+      <c r="AX83" t="inlineStr"/>
+      <c r="BY83" t="inlineStr">
+        <is>
+          <t>{"damage":12,"damage_per_card":3,"number_of_attacks":1}</t>
+        </is>
+      </c>
+      <c r="BZ83" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd":{"stat_enum":11,"is_total_stat":false,"multiplied_values":["damage"],"multiplied_values_bases":{"damage":12},"action_data":[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"damage":3,"number_of_attacks":1,"time_delay":0.0,"actions_on_lethal":[]}}]}}]</t>
+        </is>
+      </c>
+      <c r="CA83" t="inlineStr"/>
+      <c r="CB83" t="inlineStr"/>
+      <c r="CC83" t="inlineStr"/>
+      <c r="CD83" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add card reference gap A mechanics
</commit_message>
<xml_diff>
--- a/external/config/cards.xlsx
+++ b/external/config/cards.xlsx
@@ -349,7 +349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CD83"/>
+  <dimension ref="A1:CD86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -6583,27 +6583,14 @@
           <t>keyword_discard</t>
         </is>
       </c>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
       <c r="T69" t="n">
         <v>1</v>
       </c>
-      <c r="U69" t="inlineStr"/>
-      <c r="V69" t="inlineStr"/>
-      <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr"/>
-      <c r="Y69" t="inlineStr"/>
-      <c r="Z69" t="inlineStr"/>
-      <c r="AA69" t="inlineStr"/>
-      <c r="AB69" t="inlineStr"/>
-      <c r="AC69" t="inlineStr"/>
       <c r="AD69" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE69" t="inlineStr"/>
       <c r="AK69" t="n">
         <v>1</v>
       </c>
@@ -6616,7 +6603,6 @@
       <c r="AW69" t="n">
         <v>2</v>
       </c>
-      <c r="AX69" t="inlineStr"/>
       <c r="BW69" t="n">
         <v>1</v>
       </c>
@@ -6630,10 +6616,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":0,"max_card_amount":2,"card_pick_type":0,"card_pick_text":"选择最多 {0} 张牌弃掉。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionDiscardCards.gd":{}},{"res://scripts/actions/meta_actions/ActionVariableCardsetModifier.gd":{"multiplied_values":["draw_count"],"action_data":[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"draw_count":1}}]}}],"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CA69" t="inlineStr"/>
-      <c r="CB69" t="inlineStr"/>
-      <c r="CC69" t="inlineStr"/>
-      <c r="CD69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6696,48 +6678,27 @@
           <t>keyword_discard</t>
         </is>
       </c>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
-      <c r="T70" t="inlineStr"/>
-      <c r="U70" t="inlineStr"/>
-      <c r="V70" t="inlineStr"/>
-      <c r="W70" t="inlineStr"/>
-      <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr"/>
-      <c r="Z70" t="inlineStr"/>
-      <c r="AA70" t="inlineStr"/>
-      <c r="AB70" t="inlineStr"/>
-      <c r="AC70" t="inlineStr"/>
       <c r="AD70" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE70" t="inlineStr"/>
       <c r="AK70" t="n">
         <v>1</v>
       </c>
       <c r="AU70" t="n">
         <v>0</v>
       </c>
-      <c r="AV70" t="inlineStr"/>
-      <c r="AW70" t="inlineStr"/>
-      <c r="AX70" t="inlineStr"/>
       <c r="BY70" t="inlineStr">
         <is>
           <t>{"energy_amount":2}</t>
         </is>
       </c>
-      <c r="BZ70" t="inlineStr"/>
-      <c r="CA70" t="inlineStr"/>
       <c r="CB70" t="inlineStr">
         <is>
           <t>[{"res://scripts/actions/ActionAddEnergy.gd":{"energy_amount":2,"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CC70" t="inlineStr"/>
-      <c r="CD70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6795,26 +6756,11 @@
           <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
-      <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
-      <c r="T71" t="inlineStr"/>
-      <c r="U71" t="inlineStr"/>
-      <c r="V71" t="inlineStr"/>
-      <c r="W71" t="inlineStr"/>
-      <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr"/>
-      <c r="Z71" t="inlineStr"/>
-      <c r="AA71" t="inlineStr"/>
-      <c r="AB71" t="inlineStr"/>
-      <c r="AC71" t="inlineStr"/>
       <c r="AD71" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE71" t="inlineStr"/>
       <c r="AK71" t="n">
         <v>1</v>
       </c>
@@ -6830,7 +6776,6 @@
       <c r="AW71" t="n">
         <v>1</v>
       </c>
-      <c r="AX71" t="inlineStr"/>
       <c r="BY71" t="inlineStr">
         <is>
           <t>{"min_card_amount":1,"max_card_amount":1}</t>
@@ -6841,10 +6786,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"card_pick_type":4,"card_pick_text":"从弃牌堆选择 {0} 张牌。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionAddCardsToHand.gd":{}},{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd":{"card_energy_cost_until_turn":0}}],"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CA71" t="inlineStr"/>
-      <c r="CB71" t="inlineStr"/>
-      <c r="CC71" t="inlineStr"/>
-      <c r="CD71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6902,26 +6843,11 @@
           <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
-      <c r="T72" t="inlineStr"/>
-      <c r="U72" t="inlineStr"/>
-      <c r="V72" t="inlineStr"/>
-      <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
-      <c r="Z72" t="inlineStr"/>
-      <c r="AA72" t="inlineStr"/>
-      <c r="AB72" t="inlineStr"/>
-      <c r="AC72" t="inlineStr"/>
       <c r="AD72" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE72" t="inlineStr"/>
       <c r="AK72" t="n">
         <v>1</v>
       </c>
@@ -6937,7 +6863,6 @@
       <c r="AW72" t="n">
         <v>1</v>
       </c>
-      <c r="AX72" t="inlineStr"/>
       <c r="BY72" t="inlineStr">
         <is>
           <t>{"min_card_amount":1,"max_card_amount":1}</t>
@@ -6948,10 +6873,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"random_selection":true,"card_pick_type":4,"action_data":[{"res://scripts/actions/cardset_actions/ActionPlayCards.gd":{}}],"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CA72" t="inlineStr"/>
-      <c r="CB72" t="inlineStr"/>
-      <c r="CC72" t="inlineStr"/>
-      <c r="CD72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7009,20 +6930,9 @@
           <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
-      <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
       <c r="T73" t="n">
         <v>1</v>
       </c>
-      <c r="U73" t="inlineStr"/>
-      <c r="V73" t="inlineStr"/>
-      <c r="W73" t="inlineStr"/>
-      <c r="X73" t="inlineStr"/>
-      <c r="Y73" t="inlineStr"/>
-      <c r="Z73" t="inlineStr"/>
-      <c r="AA73" t="inlineStr"/>
       <c r="AB73" t="n">
         <v>1</v>
       </c>
@@ -7034,7 +6944,6 @@
           <t>""</t>
         </is>
       </c>
-      <c r="AE73" t="inlineStr"/>
       <c r="AK73" t="n">
         <v>1</v>
       </c>
@@ -7044,9 +6953,6 @@
       <c r="AU73" t="n">
         <v>0</v>
       </c>
-      <c r="AV73" t="inlineStr"/>
-      <c r="AW73" t="inlineStr"/>
-      <c r="AX73" t="inlineStr"/>
       <c r="BY73" t="inlineStr">
         <is>
           <t>{"draw_count":1,"random_consumable":1,"fill_all_slots":0}</t>
@@ -7057,10 +6963,6 @@
           <t>[{"res://scripts/actions/player_actions/ActionAddConsumable.gd":{"random_consumable":1,"fill_all_slots":0,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/ValidatorCombatStats.gd":{"stat_enum":13,"is_total_stat":false,"operator":"&gt;","comparison_value":0}}],"passed_action_data":[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
         </is>
       </c>
-      <c r="CA73" t="inlineStr"/>
-      <c r="CB73" t="inlineStr"/>
-      <c r="CC73" t="inlineStr"/>
-      <c r="CD73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7123,29 +7025,17 @@
           <t>keyword_block</t>
         </is>
       </c>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr"/>
       <c r="S74" t="n">
         <v>6</v>
       </c>
       <c r="T74" t="n">
         <v>1</v>
       </c>
-      <c r="U74" t="inlineStr"/>
-      <c r="V74" t="inlineStr"/>
-      <c r="W74" t="inlineStr"/>
-      <c r="X74" t="inlineStr"/>
-      <c r="Y74" t="inlineStr"/>
-      <c r="Z74" t="inlineStr"/>
-      <c r="AA74" t="inlineStr"/>
-      <c r="AB74" t="inlineStr"/>
-      <c r="AC74" t="inlineStr"/>
       <c r="AD74" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE74" t="inlineStr"/>
       <c r="AK74" t="n">
         <v>1</v>
       </c>
@@ -7155,9 +7045,6 @@
       <c r="AU74" t="n">
         <v>0</v>
       </c>
-      <c r="AV74" t="inlineStr"/>
-      <c r="AW74" t="inlineStr"/>
-      <c r="AX74" t="inlineStr"/>
       <c r="BY74" t="inlineStr">
         <is>
           <t>{"block":6,"draw_count":1}</t>
@@ -7168,10 +7055,6 @@
           <t>[{"res://scripts/actions/ActionBlock.gd":{"time_delay":0.5,"target_override":1,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/ValidatorCombatStats.gd":{"stat_enum":11,"is_total_stat":false,"operator":"==","comparison_value":0}}],"passed_action_data":[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"draw_count":1}}],"failed_action_data":[]}}]</t>
         </is>
       </c>
-      <c r="CA74" t="inlineStr"/>
-      <c r="CB74" t="inlineStr"/>
-      <c r="CC74" t="inlineStr"/>
-      <c r="CD74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7240,29 +7123,19 @@
       <c r="R75" t="n">
         <v>1</v>
       </c>
-      <c r="S75" t="inlineStr"/>
-      <c r="T75" t="inlineStr"/>
       <c r="U75" t="n">
         <v>4</v>
       </c>
-      <c r="V75" t="inlineStr"/>
-      <c r="W75" t="inlineStr"/>
-      <c r="X75" t="inlineStr"/>
-      <c r="Y75" t="inlineStr"/>
       <c r="Z75" t="inlineStr">
         <is>
           <t>status_effect_corrosion</t>
         </is>
       </c>
-      <c r="AA75" t="inlineStr"/>
-      <c r="AB75" t="inlineStr"/>
-      <c r="AC75" t="inlineStr"/>
       <c r="AD75" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE75" t="inlineStr"/>
       <c r="AK75" t="n">
         <v>1</v>
       </c>
@@ -7275,9 +7148,6 @@
       <c r="AU75" t="n">
         <v>0</v>
       </c>
-      <c r="AV75" t="inlineStr"/>
-      <c r="AW75" t="inlineStr"/>
-      <c r="AX75" t="inlineStr"/>
       <c r="BY75" t="inlineStr">
         <is>
           <t>{"damage":5,"number_of_attacks":1,"status_charge_amount":4,"status_effect_object_id":"status_effect_corrosion"}</t>
@@ -7288,10 +7158,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"time_delay":0.0,"actions_on_lethal":[]}},{"res://scripts/actions/status_actions/ActionApplyStatus.gd":{"time_delay":0.5,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd":{}}],"passed_action_data":[{"res://scripts/actions/enemy_actions/ActionCycleEnemyIntent.gd":{"time_delay":0.0,"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
         </is>
       </c>
-      <c r="CA75" t="inlineStr"/>
-      <c r="CB75" t="inlineStr"/>
-      <c r="CC75" t="inlineStr"/>
-      <c r="CD75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7349,26 +7215,11 @@
           <t>external/sprites/cards/green/card_green.png</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr"/>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
-      <c r="S76" t="inlineStr"/>
-      <c r="T76" t="inlineStr"/>
-      <c r="U76" t="inlineStr"/>
-      <c r="V76" t="inlineStr"/>
-      <c r="W76" t="inlineStr"/>
-      <c r="X76" t="inlineStr"/>
-      <c r="Y76" t="inlineStr"/>
-      <c r="Z76" t="inlineStr"/>
-      <c r="AA76" t="inlineStr"/>
-      <c r="AB76" t="inlineStr"/>
-      <c r="AC76" t="inlineStr"/>
       <c r="AD76" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE76" t="inlineStr"/>
       <c r="AK76" t="n">
         <v>1</v>
       </c>
@@ -7381,7 +7232,6 @@
       <c r="AW76" t="n">
         <v>1</v>
       </c>
-      <c r="AX76" t="inlineStr"/>
       <c r="BY76" t="inlineStr">
         <is>
           <t>{"improve_amount":2,"min_card_amount":1,"max_card_amount":1}</t>
@@ -7392,10 +7242,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"card_pick_type":0,"card_pick_text":"选择 {0} 张牌调音。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd":{"improve_parent_card":false,"card_value_improvements":{"damage":2,"block":2}}}],"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CA76" t="inlineStr"/>
-      <c r="CB76" t="inlineStr"/>
-      <c r="CC76" t="inlineStr"/>
-      <c r="CD76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7458,27 +7304,14 @@
           <t>keyword_block,keyword_retain</t>
         </is>
       </c>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
         <v>6</v>
       </c>
-      <c r="T77" t="inlineStr"/>
-      <c r="U77" t="inlineStr"/>
-      <c r="V77" t="inlineStr"/>
-      <c r="W77" t="inlineStr"/>
-      <c r="X77" t="inlineStr"/>
-      <c r="Y77" t="inlineStr"/>
-      <c r="Z77" t="inlineStr"/>
-      <c r="AA77" t="inlineStr"/>
-      <c r="AB77" t="inlineStr"/>
-      <c r="AC77" t="inlineStr"/>
       <c r="AD77" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE77" t="inlineStr"/>
       <c r="AK77" t="n">
         <v>1</v>
       </c>
@@ -7488,9 +7321,6 @@
       <c r="AU77" t="n">
         <v>0</v>
       </c>
-      <c r="AV77" t="inlineStr"/>
-      <c r="AW77" t="inlineStr"/>
-      <c r="AX77" t="inlineStr"/>
       <c r="BY77" t="inlineStr">
         <is>
           <t>{"block":6,"improve_amount":2}</t>
@@ -7501,14 +7331,11 @@
           <t>[{"res://scripts/actions/ActionBlock.gd":{"time_delay":0.5,"target_override":1,"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CA77" t="inlineStr"/>
-      <c r="CB77" t="inlineStr"/>
       <c r="CC77" t="inlineStr">
         <is>
           <t>[{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd":{"pick_played_card":true,"improve_parent_card":false,"card_value_improvements":{"block":2}}}]</t>
         </is>
       </c>
-      <c r="CD77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7571,27 +7398,14 @@
           <t>keyword_exhaust</t>
         </is>
       </c>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr"/>
-      <c r="S78" t="inlineStr"/>
       <c r="T78" t="n">
         <v>1</v>
       </c>
-      <c r="U78" t="inlineStr"/>
-      <c r="V78" t="inlineStr"/>
-      <c r="W78" t="inlineStr"/>
-      <c r="X78" t="inlineStr"/>
-      <c r="Y78" t="inlineStr"/>
-      <c r="Z78" t="inlineStr"/>
-      <c r="AA78" t="inlineStr"/>
-      <c r="AB78" t="inlineStr"/>
-      <c r="AC78" t="inlineStr"/>
       <c r="AD78" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE78" t="inlineStr"/>
       <c r="AK78" t="n">
         <v>1</v>
       </c>
@@ -7601,9 +7415,6 @@
       <c r="AU78" t="n">
         <v>0</v>
       </c>
-      <c r="AV78" t="inlineStr"/>
-      <c r="AW78" t="inlineStr"/>
-      <c r="AX78" t="inlineStr"/>
       <c r="BY78" t="inlineStr">
         <is>
           <t>{"energy_amount":1,"draw_count":1}</t>
@@ -7619,9 +7430,6 @@
           <t>[{"res://scripts/actions/ActionAddEnergy.gd":{"energy_amount":1,"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CB78" t="inlineStr"/>
-      <c r="CC78" t="inlineStr"/>
-      <c r="CD78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7679,30 +7487,17 @@
           <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr"/>
       <c r="Q79" t="n">
         <v>7</v>
       </c>
       <c r="R79" t="n">
         <v>1</v>
       </c>
-      <c r="S79" t="inlineStr"/>
-      <c r="T79" t="inlineStr"/>
-      <c r="U79" t="inlineStr"/>
-      <c r="V79" t="inlineStr"/>
-      <c r="W79" t="inlineStr"/>
-      <c r="X79" t="inlineStr"/>
-      <c r="Y79" t="inlineStr"/>
-      <c r="Z79" t="inlineStr"/>
-      <c r="AA79" t="inlineStr"/>
-      <c r="AB79" t="inlineStr"/>
-      <c r="AC79" t="inlineStr"/>
       <c r="AD79" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE79" t="inlineStr"/>
       <c r="AK79" t="n">
         <v>1</v>
       </c>
@@ -7712,9 +7507,6 @@
       <c r="AU79" t="n">
         <v>0</v>
       </c>
-      <c r="AV79" t="inlineStr"/>
-      <c r="AW79" t="inlineStr"/>
-      <c r="AX79" t="inlineStr"/>
       <c r="BY79" t="inlineStr">
         <is>
           <t>{"damage":7,"bonus_damage":8,"number_of_attacks":1}</t>
@@ -7725,10 +7517,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"time_delay":0.0,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/ValidatorCombatStats.gd":{"stat_enum":14,"is_total_stat":false,"operator":"&gt;","comparison_value":0}}],"passed_action_data":[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"custom_key_names":{"damage":"bonus_damage"},"number_of_attacks":1,"time_delay":0.0,"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
         </is>
       </c>
-      <c r="CA79" t="inlineStr"/>
-      <c r="CB79" t="inlineStr"/>
-      <c r="CC79" t="inlineStr"/>
-      <c r="CD79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7791,29 +7579,17 @@
           <t>keyword_exhaust,keyword_block</t>
         </is>
       </c>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
       <c r="S80" t="n">
         <v>6</v>
       </c>
       <c r="T80" t="n">
         <v>1</v>
       </c>
-      <c r="U80" t="inlineStr"/>
-      <c r="V80" t="inlineStr"/>
-      <c r="W80" t="inlineStr"/>
-      <c r="X80" t="inlineStr"/>
-      <c r="Y80" t="inlineStr"/>
-      <c r="Z80" t="inlineStr"/>
-      <c r="AA80" t="inlineStr"/>
-      <c r="AB80" t="inlineStr"/>
-      <c r="AC80" t="inlineStr"/>
       <c r="AD80" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE80" t="inlineStr"/>
       <c r="AK80" t="n">
         <v>1</v>
       </c>
@@ -7829,7 +7605,6 @@
       <c r="AW80" t="n">
         <v>1</v>
       </c>
-      <c r="AX80" t="inlineStr"/>
       <c r="BY80" t="inlineStr">
         <is>
           <t>{"block":6,"draw_count":1,"min_card_amount":1,"max_card_amount":1}</t>
@@ -7840,10 +7615,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd":{"min_card_amount":1,"max_card_amount":1,"min_cards_are_required_for_action":true,"card_pick_type":0,"card_pick_text":"选择 {0} 张牌放逐。已选择 {1} 张牌","action_data":[{"res://scripts/actions/cardset_actions/ActionExhaustCards.gd":{}},{"res://scripts/actions/ActionBlock.gd":{"target_override":1,"time_delay":0.5}},{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd":{"draw_count":1}}],"actions_on_lethal":[]}}]</t>
         </is>
       </c>
-      <c r="CA80" t="inlineStr"/>
-      <c r="CB80" t="inlineStr"/>
-      <c r="CC80" t="inlineStr"/>
-      <c r="CD80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7901,30 +7672,17 @@
           <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr"/>
       <c r="Q81" t="n">
         <v>12</v>
       </c>
       <c r="R81" t="n">
         <v>1</v>
       </c>
-      <c r="S81" t="inlineStr"/>
-      <c r="T81" t="inlineStr"/>
-      <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr"/>
-      <c r="W81" t="inlineStr"/>
-      <c r="X81" t="inlineStr"/>
-      <c r="Y81" t="inlineStr"/>
-      <c r="Z81" t="inlineStr"/>
-      <c r="AA81" t="inlineStr"/>
-      <c r="AB81" t="inlineStr"/>
-      <c r="AC81" t="inlineStr"/>
       <c r="AD81" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE81" t="inlineStr"/>
       <c r="AK81" t="n">
         <v>1</v>
       </c>
@@ -7934,9 +7692,6 @@
       <c r="AU81" t="n">
         <v>0</v>
       </c>
-      <c r="AV81" t="inlineStr"/>
-      <c r="AW81" t="inlineStr"/>
-      <c r="AX81" t="inlineStr"/>
       <c r="BY81" t="inlineStr">
         <is>
           <t>{"damage":12,"number_of_attacks":1}</t>
@@ -7952,9 +7707,6 @@
           <t>[{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd":{"pick_played_card":true,"card_energy_cost_until_turn":0}}]</t>
         </is>
       </c>
-      <c r="CB81" t="inlineStr"/>
-      <c r="CC81" t="inlineStr"/>
-      <c r="CD81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8012,36 +7764,25 @@
           <t>external/sprites/cards/red/card_red.png</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr"/>
       <c r="Q82" t="n">
         <v>7</v>
       </c>
       <c r="R82" t="n">
         <v>1</v>
       </c>
-      <c r="S82" t="inlineStr"/>
-      <c r="T82" t="inlineStr"/>
       <c r="U82" t="n">
         <v>2</v>
       </c>
-      <c r="V82" t="inlineStr"/>
-      <c r="W82" t="inlineStr"/>
-      <c r="X82" t="inlineStr"/>
-      <c r="Y82" t="inlineStr"/>
       <c r="Z82" t="inlineStr">
         <is>
           <t>status_effect_vulnerable</t>
         </is>
       </c>
-      <c r="AA82" t="inlineStr"/>
-      <c r="AB82" t="inlineStr"/>
-      <c r="AC82" t="inlineStr"/>
       <c r="AD82" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE82" t="inlineStr"/>
       <c r="AK82" t="n">
         <v>1</v>
       </c>
@@ -8051,9 +7792,6 @@
       <c r="AU82" t="n">
         <v>0</v>
       </c>
-      <c r="AV82" t="inlineStr"/>
-      <c r="AW82" t="inlineStr"/>
-      <c r="AX82" t="inlineStr"/>
       <c r="BY82" t="inlineStr">
         <is>
           <t>{"damage":7,"number_of_attacks":1,"status_charge_amount":2,"status_effect_object_id":"status_effect_vulnerable"}</t>
@@ -8064,10 +7802,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"time_delay":0.0,"actions_on_lethal":[]}},{"res://scripts/actions/meta_actions/ActionValidator.gd":{"validator_data":[{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd":{}}],"passed_action_data":[{"res://scripts/actions/status_actions/ActionApplyStatus.gd":{"status_charge_amount":2,"status_effect_object_id":"status_effect_vulnerable","time_delay":0.5,"actions_on_lethal":[]}}],"failed_action_data":[]}}]</t>
         </is>
       </c>
-      <c r="CA82" t="inlineStr"/>
-      <c r="CB82" t="inlineStr"/>
-      <c r="CC82" t="inlineStr"/>
-      <c r="CD82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8125,30 +7859,17 @@
           <t>external/sprites/cards/red/card_red.png</t>
         </is>
       </c>
-      <c r="P83" t="inlineStr"/>
       <c r="Q83" t="n">
         <v>12</v>
       </c>
       <c r="R83" t="n">
         <v>1</v>
       </c>
-      <c r="S83" t="inlineStr"/>
-      <c r="T83" t="inlineStr"/>
-      <c r="U83" t="inlineStr"/>
-      <c r="V83" t="inlineStr"/>
-      <c r="W83" t="inlineStr"/>
-      <c r="X83" t="inlineStr"/>
-      <c r="Y83" t="inlineStr"/>
-      <c r="Z83" t="inlineStr"/>
-      <c r="AA83" t="inlineStr"/>
-      <c r="AB83" t="inlineStr"/>
-      <c r="AC83" t="inlineStr"/>
       <c r="AD83" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="AE83" t="inlineStr"/>
       <c r="AK83" t="n">
         <v>1</v>
       </c>
@@ -8158,9 +7879,6 @@
       <c r="AU83" t="n">
         <v>0</v>
       </c>
-      <c r="AV83" t="inlineStr"/>
-      <c r="AW83" t="inlineStr"/>
-      <c r="AX83" t="inlineStr"/>
       <c r="BY83" t="inlineStr">
         <is>
           <t>{"damage":12,"damage_per_card":3,"number_of_attacks":1}</t>
@@ -8171,10 +7889,488 @@
           <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd":{"stat_enum":11,"is_total_stat":false,"multiplied_values":["damage"],"multiplied_values_bases":{"damage":12},"action_data":[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd":{"damage":3,"number_of_attacks":1,"time_delay":0.0,"actions_on_lethal":[]}}]}}]</t>
         </is>
       </c>
-      <c r="CA83" t="inlineStr"/>
-      <c r="CB83" t="inlineStr"/>
-      <c r="CC83" t="inlineStr"/>
-      <c r="CD83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>card_pursuit</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>追击</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>造成 [damage] 点伤害。若上一张牌是攻击，抽 [draw_count] 张牌。</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="n">
+        <v>1</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>color_red</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J84" t="b">
+        <v>1</v>
+      </c>
+      <c r="K84" t="b">
+        <v>0</v>
+      </c>
+      <c r="L84" t="b">
+        <v>0</v>
+      </c>
+      <c r="M84" t="b">
+        <v>0</v>
+      </c>
+      <c r="N84" t="b">
+        <v>1</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/red/card_red.png</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="n">
+        <v>6</v>
+      </c>
+      <c r="R84" t="n">
+        <v>1</v>
+      </c>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="n">
+        <v>1</v>
+      </c>
+      <c r="U84" t="inlineStr"/>
+      <c r="V84" t="inlineStr"/>
+      <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr"/>
+      <c r="Y84" t="inlineStr"/>
+      <c r="Z84" t="inlineStr"/>
+      <c r="AA84" t="inlineStr"/>
+      <c r="AB84" t="inlineStr"/>
+      <c r="AC84" t="inlineStr"/>
+      <c r="AD84" t="inlineStr"/>
+      <c r="AE84" t="inlineStr"/>
+      <c r="AF84" t="inlineStr"/>
+      <c r="AG84" t="inlineStr"/>
+      <c r="AH84" t="inlineStr"/>
+      <c r="AI84" t="inlineStr"/>
+      <c r="AJ84" t="inlineStr"/>
+      <c r="AK84" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL84" t="inlineStr"/>
+      <c r="AM84" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN84" t="inlineStr"/>
+      <c r="AO84" t="inlineStr"/>
+      <c r="AP84" t="inlineStr"/>
+      <c r="AQ84" t="inlineStr"/>
+      <c r="AR84" t="inlineStr"/>
+      <c r="AS84" t="inlineStr"/>
+      <c r="AT84" t="inlineStr"/>
+      <c r="AU84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV84" t="inlineStr"/>
+      <c r="AW84" t="inlineStr"/>
+      <c r="AX84" t="inlineStr"/>
+      <c r="AY84" t="inlineStr"/>
+      <c r="AZ84" t="inlineStr"/>
+      <c r="BA84" t="inlineStr"/>
+      <c r="BB84" t="inlineStr"/>
+      <c r="BC84" t="inlineStr"/>
+      <c r="BD84" t="inlineStr"/>
+      <c r="BE84" t="inlineStr"/>
+      <c r="BF84" t="inlineStr"/>
+      <c r="BG84" t="inlineStr"/>
+      <c r="BH84" t="inlineStr"/>
+      <c r="BI84" t="inlineStr"/>
+      <c r="BJ84" t="inlineStr"/>
+      <c r="BK84" t="inlineStr"/>
+      <c r="BL84" t="inlineStr"/>
+      <c r="BM84" t="inlineStr"/>
+      <c r="BN84" t="inlineStr"/>
+      <c r="BO84" t="inlineStr"/>
+      <c r="BP84" t="inlineStr"/>
+      <c r="BQ84" t="inlineStr"/>
+      <c r="BR84" t="inlineStr"/>
+      <c r="BS84" t="inlineStr"/>
+      <c r="BT84" t="inlineStr"/>
+      <c r="BU84" t="inlineStr"/>
+      <c r="BV84" t="inlineStr"/>
+      <c r="BW84" t="inlineStr"/>
+      <c r="BX84" t="inlineStr"/>
+      <c r="BY84" t="inlineStr">
+        <is>
+          <t>{"damage": 6, "number_of_attacks": 1, "draw_count": 1}</t>
+        </is>
+      </c>
+      <c r="BZ84" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "failed_action_data": []}}]</t>
+        </is>
+      </c>
+      <c r="CA84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CB84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CC84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CD84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>card_echo_shield</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>回声护盾</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>获得 [block] 点格挡。若上一张牌也是技能，额外获得 [bonus_block] 点格挡。</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J85" t="b">
+        <v>0</v>
+      </c>
+      <c r="K85" t="b">
+        <v>0</v>
+      </c>
+      <c r="L85" t="b">
+        <v>0</v>
+      </c>
+      <c r="M85" t="b">
+        <v>0</v>
+      </c>
+      <c r="N85" t="b">
+        <v>1</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>keyword_block</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="n">
+        <v>7</v>
+      </c>
+      <c r="T85" t="inlineStr"/>
+      <c r="U85" t="inlineStr"/>
+      <c r="V85" t="inlineStr"/>
+      <c r="W85" t="inlineStr"/>
+      <c r="X85" t="inlineStr"/>
+      <c r="Y85" t="inlineStr"/>
+      <c r="Z85" t="inlineStr"/>
+      <c r="AA85" t="inlineStr"/>
+      <c r="AB85" t="inlineStr"/>
+      <c r="AC85" t="inlineStr"/>
+      <c r="AD85" t="inlineStr"/>
+      <c r="AE85" t="inlineStr"/>
+      <c r="AF85" t="inlineStr"/>
+      <c r="AG85" t="inlineStr"/>
+      <c r="AH85" t="inlineStr"/>
+      <c r="AI85" t="inlineStr"/>
+      <c r="AJ85" t="inlineStr"/>
+      <c r="AK85" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL85" t="inlineStr"/>
+      <c r="AM85" t="inlineStr"/>
+      <c r="AN85" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO85" t="inlineStr"/>
+      <c r="AP85" t="inlineStr"/>
+      <c r="AQ85" t="inlineStr"/>
+      <c r="AR85" t="inlineStr"/>
+      <c r="AS85" t="inlineStr"/>
+      <c r="AT85" t="inlineStr"/>
+      <c r="AU85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV85" t="inlineStr"/>
+      <c r="AW85" t="inlineStr"/>
+      <c r="AX85" t="inlineStr"/>
+      <c r="AY85" t="inlineStr"/>
+      <c r="AZ85" t="inlineStr"/>
+      <c r="BA85" t="inlineStr"/>
+      <c r="BB85" t="inlineStr"/>
+      <c r="BC85" t="inlineStr"/>
+      <c r="BD85" t="inlineStr"/>
+      <c r="BE85" t="inlineStr"/>
+      <c r="BF85" t="inlineStr"/>
+      <c r="BG85" t="inlineStr"/>
+      <c r="BH85" t="inlineStr"/>
+      <c r="BI85" t="inlineStr"/>
+      <c r="BJ85" t="inlineStr"/>
+      <c r="BK85" t="inlineStr"/>
+      <c r="BL85" t="inlineStr"/>
+      <c r="BM85" t="inlineStr"/>
+      <c r="BN85" t="inlineStr"/>
+      <c r="BO85" t="inlineStr"/>
+      <c r="BP85" t="inlineStr"/>
+      <c r="BQ85" t="inlineStr"/>
+      <c r="BR85" t="inlineStr"/>
+      <c r="BS85" t="inlineStr"/>
+      <c r="BT85" t="inlineStr"/>
+      <c r="BU85" t="inlineStr"/>
+      <c r="BV85" t="inlineStr"/>
+      <c r="BW85" t="inlineStr"/>
+      <c r="BX85" t="inlineStr"/>
+      <c r="BY85" t="inlineStr">
+        <is>
+          <t>{"block": 7, "bonus_block": 6}</t>
+        </is>
+      </c>
+      <c r="BZ85" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 1}}], "passed_action_data": [{"res://scripts/actions/ActionBlock.gd": {"custom_key_names": {"block": "bonus_block"}, "time_delay": 0.5, "target_override": 1}}], "failed_action_data": []}}]</t>
+        </is>
+      </c>
+      <c r="CA85" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CB85" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CC85" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CD85" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>card_finale_burst</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>终场爆音</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>造成 [damage] 点伤害。目标每有1层腐蚀，额外造成 [corrosion_damage_multiplier] 点伤害。</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
+        <v>3</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>2</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J86" t="b">
+        <v>1</v>
+      </c>
+      <c r="K86" t="b">
+        <v>0</v>
+      </c>
+      <c r="L86" t="b">
+        <v>0</v>
+      </c>
+      <c r="M86" t="b">
+        <v>0</v>
+      </c>
+      <c r="N86" t="b">
+        <v>1</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>keyword_corrosion</t>
+        </is>
+      </c>
+      <c r="Q86" t="n">
+        <v>8</v>
+      </c>
+      <c r="R86" t="n">
+        <v>1</v>
+      </c>
+      <c r="S86" t="inlineStr"/>
+      <c r="T86" t="inlineStr"/>
+      <c r="U86" t="inlineStr"/>
+      <c r="V86" t="inlineStr"/>
+      <c r="W86" t="inlineStr"/>
+      <c r="X86" t="inlineStr"/>
+      <c r="Y86" t="inlineStr"/>
+      <c r="Z86" t="inlineStr"/>
+      <c r="AA86" t="inlineStr"/>
+      <c r="AB86" t="inlineStr"/>
+      <c r="AC86" t="inlineStr"/>
+      <c r="AD86" t="inlineStr"/>
+      <c r="AE86" t="inlineStr"/>
+      <c r="AF86" t="inlineStr"/>
+      <c r="AG86" t="inlineStr"/>
+      <c r="AH86" t="inlineStr"/>
+      <c r="AI86" t="inlineStr"/>
+      <c r="AJ86" t="inlineStr"/>
+      <c r="AK86" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL86" t="inlineStr"/>
+      <c r="AM86" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN86" t="inlineStr"/>
+      <c r="AO86" t="inlineStr"/>
+      <c r="AP86" t="inlineStr"/>
+      <c r="AQ86" t="inlineStr"/>
+      <c r="AR86" t="inlineStr"/>
+      <c r="AS86" t="inlineStr"/>
+      <c r="AT86" t="inlineStr"/>
+      <c r="AU86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV86" t="inlineStr"/>
+      <c r="AW86" t="inlineStr"/>
+      <c r="AX86" t="inlineStr"/>
+      <c r="AY86" t="inlineStr"/>
+      <c r="AZ86" t="inlineStr"/>
+      <c r="BA86" t="inlineStr"/>
+      <c r="BB86" t="inlineStr"/>
+      <c r="BC86" t="inlineStr"/>
+      <c r="BD86" t="inlineStr"/>
+      <c r="BE86" t="inlineStr"/>
+      <c r="BF86" t="inlineStr"/>
+      <c r="BG86" t="inlineStr"/>
+      <c r="BH86" t="inlineStr"/>
+      <c r="BI86" t="inlineStr"/>
+      <c r="BJ86" t="inlineStr"/>
+      <c r="BK86" t="inlineStr"/>
+      <c r="BL86" t="inlineStr"/>
+      <c r="BM86" t="inlineStr"/>
+      <c r="BN86" t="inlineStr"/>
+      <c r="BO86" t="inlineStr"/>
+      <c r="BP86" t="inlineStr"/>
+      <c r="BQ86" t="inlineStr"/>
+      <c r="BR86" t="inlineStr"/>
+      <c r="BS86" t="inlineStr"/>
+      <c r="BT86" t="inlineStr"/>
+      <c r="BU86" t="inlineStr"/>
+      <c r="BV86" t="inlineStr"/>
+      <c r="BW86" t="inlineStr"/>
+      <c r="BX86" t="inlineStr"/>
+      <c r="BY86" t="inlineStr">
+        <is>
+          <t>{"damage": 8, "corrosion_damage_multiplier": 2, "number_of_attacks": 1}</t>
+        </is>
+      </c>
+      <c r="BZ86" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/meta_actions/ActionTargetStatusValueModifier.gd": {"status_effect_object_id": "status_effect_corrosion", "charge_key": "status_charges", "multiplier": 2, "value_key": "damage", "operation": "add", "default_value": 0, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
+        </is>
+      </c>
+      <c r="CA86" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CB86" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CC86" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="CD86" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update card ledger for combo starter
</commit_message>
<xml_diff>
--- a/external/config/cards.xlsx
+++ b/external/config/cards.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA23"/>
+  <dimension ref="A1:BA24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1181,28 +1181,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>card_distorted_note</t>
+          <t>card_combo_starter</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>失真音</t>
+          <t>连段起手</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>造成 [damage] 点伤害并施加 [status_charge_amount] 层腐蚀。如果目标正在攻击，切换其意图。</t>
+          <t>你的下一张攻击造成额外 [damage] 点伤害。</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>color_green</t>
+          <t>color_red</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -1215,7 +1215,7 @@
         <v>-1</v>
       </c>
       <c r="J6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" t="b">
         <v>0</v>
@@ -1231,34 +1231,22 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>external/sprites/cards/green/card_green.png</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>keyword_corrosion</t>
-        </is>
-      </c>
+          <t>external/sprites/cards/red/card_red.png</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R6" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="n">
-        <v>4</v>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>status_effect_corrosion</t>
-        </is>
-      </c>
+      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
@@ -1266,13 +1254,15 @@
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>ActionAttackGenerator</t>
-        </is>
-      </c>
-      <c r="AG6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH6" t="inlineStr"/>
+          <t>ActionApplyStatus</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
+        </is>
+      </c>
       <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="n">
@@ -1285,9 +1275,7 @@
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="n">
-        <v>2</v>
-      </c>
+      <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr"/>
@@ -1296,12 +1284,12 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>{"damage": 5, "number_of_attacks": 1, "status_charge_amount": 4, "status_effect_object_id": "status_effect_corrosion"}</t>
+          <t>{"damage": 3}</t>
         </is>
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"time_delay": 0.5, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd": {}}], "passed_action_data": [{"res://scripts/actions/enemy_actions/ActionCycleEnemyIntent.gd": {"time_delay": 0.0, "actions_on_lethal": []}}], "failed_action_data": []}}]</t>
+          <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_combo_starter", "status_charge_amount": 1, "status_custom_values": {"card_type_filter": [0], "value_modifiers": {"damage": 3}, "consume_charge_on_trigger": true, "clear_on_player_turn_end": true, "ignore_duplicate_plays": true}}}]</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -1312,21 +1300,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>card_echo_shield</t>
+          <t>card_distorted_note</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>回声护盾</t>
+          <t>失真音</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>获得 [block] 点格挡。若上一张牌也是技能，额外获得 [bonus_block] 点格挡。</t>
+          <t>造成 [damage] 点伤害并施加 [status_charge_amount] 层腐蚀。如果目标正在攻击，切换其意图。</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
@@ -1346,7 +1334,7 @@
         <v>-1</v>
       </c>
       <c r="J7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="b">
         <v>0</v>
@@ -1367,21 +1355,29 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>keyword_block</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="n">
-        <v>7</v>
-      </c>
+          <t>keyword_corrosion</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>5</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="n">
+        <v>4</v>
+      </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>status_effect_corrosion</t>
+        </is>
+      </c>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
@@ -1389,30 +1385,28 @@
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>ActionBlock</t>
+          <t>ActionAttackGenerator</t>
         </is>
       </c>
       <c r="AG7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="n">
         <v>1</v>
       </c>
       <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="n">
-        <v>3</v>
-      </c>
+      <c r="AM7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
+      <c r="AQ7" t="n">
+        <v>2</v>
+      </c>
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
@@ -1421,12 +1415,12 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>{"block": 7, "bonus_block": 6}</t>
+          <t>{"damage": 5, "number_of_attacks": 1, "status_charge_amount": 4, "status_effect_object_id": "status_effect_corrosion"}</t>
         </is>
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 1}}], "passed_action_data": [{"res://scripts/actions/ActionBlock.gd": {"custom_key_names": {"block": "bonus_block"}, "time_delay": 0.5, "target_override": 1}}], "failed_action_data": []}}]</t>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"time_delay": 0.5, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd": {}}], "passed_action_data": [{"res://scripts/actions/enemy_actions/ActionCycleEnemyIntent.gd": {"time_delay": 0.0, "actions_on_lethal": []}}], "failed_action_data": []}}]</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr"/>
@@ -1437,24 +1431,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>card_finale_burst</t>
+          <t>card_echo_shield</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>终场爆音</t>
+          <t>回声护盾</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>造成 [damage] 点伤害。目标每有1层腐蚀，额外造成 [corrosion_damage_multiplier] 点伤害。</t>
+          <t>获得 [block] 点格挡。若上一张牌也是技能，额外获得 [bonus_block] 点格挡。</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1462,7 +1456,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -1471,7 +1465,7 @@
         <v>-1</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="b">
         <v>0</v>
@@ -1492,16 +1486,14 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>keyword_corrosion</t>
-        </is>
-      </c>
-      <c r="Q8" t="n">
-        <v>8</v>
-      </c>
-      <c r="R8" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>keyword_block</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>7</v>
+      </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
@@ -1516,21 +1508,27 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>ActionTargetStatusValueModifier</t>
-        </is>
-      </c>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
+          <t>ActionBlock</t>
+        </is>
+      </c>
+      <c r="AG8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
+        </is>
+      </c>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="n">
         <v>1</v>
       </c>
       <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="n">
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="n">
         <v>3</v>
       </c>
-      <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr"/>
@@ -1542,12 +1540,12 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>{"damage": 8, "corrosion_damage_multiplier": 2, "number_of_attacks": 1}</t>
+          <t>{"block": 7, "bonus_block": 6}</t>
         </is>
       </c>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionTargetStatusValueModifier.gd": {"status_effect_object_id": "status_effect_corrosion", "charge_key": "status_charges", "multiplier": 2, "value_key": "damage", "operation": "add", "default_value": 0, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
+          <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 1}}], "passed_action_data": [{"res://scripts/actions/ActionBlock.gd": {"custom_key_names": {"block": "bonus_block"}, "time_delay": 0.5, "target_override": 1}}], "failed_action_data": []}}]</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr"/>
@@ -1558,17 +1556,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>card_finisher</t>
+          <t>card_finale_burst</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>终结拳</t>
+          <t>终场爆音</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>造成 [damage] 点伤害。本回合每打出过1张牌，额外造成 [damage_per_card] 点伤害。</t>
+          <t>造成 [damage] 点伤害。目标每有1层腐蚀，额外造成 [corrosion_damage_multiplier] 点伤害。</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1579,7 +1577,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>color_red</t>
+          <t>color_green</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -1608,12 +1606,16 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>external/sprites/cards/red/card_red.png</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr"/>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>keyword_corrosion</t>
+        </is>
+      </c>
       <c r="Q9" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="R9" t="n">
         <v>1</v>
@@ -1633,7 +1635,7 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>ActionVariableCombatStatsModifier</t>
+          <t>ActionTargetStatusValueModifier</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr"/>
@@ -1643,10 +1645,10 @@
       <c r="AK9" t="n">
         <v>1</v>
       </c>
-      <c r="AL9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="n">
+        <v>3</v>
+      </c>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
@@ -1659,12 +1661,12 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>{"damage": 12, "damage_per_card": 3, "number_of_attacks": 1}</t>
+          <t>{"damage": 8, "corrosion_damage_multiplier": 2, "number_of_attacks": 1}</t>
         </is>
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd": {"stat_enum": 11, "is_total_stat": false, "multiplied_values": ["damage"], "multiplied_values_bases": {"damage": 12}, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"damage": 3, "number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
+          <t>[{"res://scripts/actions/meta_actions/ActionTargetStatusValueModifier.gd": {"status_effect_object_id": "status_effect_corrosion", "charge_key": "status_charges", "multiplier": 2, "value_key": "damage", "operation": "add", "default_value": 0, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr"/>
@@ -1675,32 +1677,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>card_first_beat</t>
+          <t>card_finisher</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>第一拍</t>
+          <t>终结拳</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>获得 [block] 点格挡。如果这是本回合打出的第一张牌，额外抽 [draw_count] 张牌。</t>
+          <t>造成 [damage] 点伤害。本回合每打出过1张牌，额外造成 [damage_per_card] 点伤害。</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>color_green</t>
+          <t>color_red</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -1709,7 +1711,7 @@
         <v>-1</v>
       </c>
       <c r="J10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="b">
         <v>0</v>
@@ -1725,22 +1727,18 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>external/sprites/cards/green/card_green.png</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>keyword_block</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="n">
-        <v>6</v>
-      </c>
-      <c r="T10" t="n">
-        <v>1</v>
-      </c>
+          <t>external/sprites/cards/red/card_red.png</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="n">
+        <v>12</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
@@ -1754,27 +1752,21 @@
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>ActionBlock</t>
-        </is>
-      </c>
-      <c r="AG10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
-        </is>
-      </c>
+          <t>ActionVariableCombatStatsModifier</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="n">
         <v>1</v>
       </c>
-      <c r="AL10" t="inlineStr"/>
+      <c r="AL10" t="n">
+        <v>1</v>
+      </c>
       <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="n">
-        <v>3</v>
-      </c>
+      <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
       <c r="AQ10" t="inlineStr"/>
@@ -1786,12 +1778,12 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>{"block": 6, "draw_count": 1}</t>
+          <t>{"damage": 12, "damage_per_card": 3, "number_of_attacks": 1}</t>
         </is>
       </c>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/ValidatorCombatStats.gd": {"stat_enum": 11, "is_total_stat": false, "operator": "==", "comparison_value": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "failed_action_data": []}}]</t>
+          <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd": {"stat_enum": 11, "is_total_stat": false, "multiplied_values": ["damage"], "multiplied_values_bases": {"damage": 12}, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"damage": 3, "number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr"/>
@@ -1802,17 +1794,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>card_hasty_sorting</t>
+          <t>card_first_beat</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>慌忙整理</t>
+          <t>第一拍</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>弃置最多 [max_card_amount] 张牌。每弃置1张，抽 [draw_count] 张牌。</t>
+          <t>获得 [block] 点格挡。如果这是本回合打出的第一张牌，额外抽 [draw_count] 张牌。</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1823,7 +1815,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>color_blue</t>
+          <t>color_green</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -1852,17 +1844,19 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>external/sprites/cards/blue/card_blue.png</t>
+          <t>external/sprites/cards/green/card_green.png</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>keyword_discard</t>
+          <t>keyword_block</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>6</v>
+      </c>
       <c r="T11" t="n">
         <v>1</v>
       </c>
@@ -1879,11 +1873,17 @@
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>ActionPickCards</t>
-        </is>
-      </c>
-      <c r="AG11" t="inlineStr"/>
-      <c r="AH11" t="inlineStr"/>
+          <t>ActionBlock</t>
+        </is>
+      </c>
+      <c r="AG11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
+        </is>
+      </c>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="n">
@@ -1891,7 +1891,9 @@
       </c>
       <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="inlineStr"/>
-      <c r="AN11" t="inlineStr"/>
+      <c r="AN11" t="n">
+        <v>3</v>
+      </c>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="inlineStr"/>
@@ -1903,12 +1905,12 @@
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>{"draw_count": 1, "min_card_amount": 0, "max_card_amount": 2}</t>
+          <t>{"block": 6, "draw_count": 1}</t>
         </is>
       </c>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 0, "max_card_amount": 2, "card_pick_type": 0, "card_pick_text": "选择最多 {0} 张牌弃掉。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionDiscardCards.gd": {}}, {"res://scripts/actions/meta_actions/ActionVariableCardsetModifier.gd": {"multiplied_values": ["draw_count"], "action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}]}}], "actions_on_lethal": []}}]</t>
+          <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/ValidatorCombatStats.gd": {"stat_enum": 11, "is_total_stat": false, "operator": "==", "comparison_value": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "failed_action_data": []}}]</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr"/>
@@ -1919,32 +1921,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>card_last_item</t>
+          <t>card_hasty_sorting</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>最后一件</t>
+          <t>慌忙整理</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>造成 [damage] 点伤害。本场战斗每消耗过1张牌，额外造成 [damage_per_exhaust] 点伤害。</t>
+          <t>弃置最多 [max_card_amount] 张牌。每弃置1张，抽 [draw_count] 张牌。</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>color_orange</t>
+          <t>color_blue</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
@@ -1953,7 +1955,7 @@
         <v>-1</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
@@ -1969,18 +1971,20 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>external/sprites/cards/orange/card_orange.png</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="n">
-        <v>10</v>
-      </c>
-      <c r="R12" t="n">
-        <v>1</v>
-      </c>
+          <t>external/sprites/cards/blue/card_blue.png</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>keyword_discard</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
@@ -1994,7 +1998,7 @@
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>ActionVariableCombatStatsModifier</t>
+          <t>ActionPickCards</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr"/>
@@ -2004,9 +2008,7 @@
       <c r="AK12" t="n">
         <v>1</v>
       </c>
-      <c r="AL12" t="n">
-        <v>1</v>
-      </c>
+      <c r="AL12" t="inlineStr"/>
       <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
@@ -2020,12 +2022,12 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>{"damage": 10, "damage_per_exhaust": 2, "number_of_attacks": 1}</t>
+          <t>{"draw_count": 1, "min_card_amount": 0, "max_card_amount": 2}</t>
         </is>
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd": {"stat_enum": 14, "is_total_stat": true, "multiplied_values": ["damage"], "multiplied_values_bases": {"damage": 10}, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"damage": 2, "number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 0, "max_card_amount": 2, "card_pick_type": 0, "card_pick_text": "选择最多 {0} 张牌弃掉。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionDiscardCards.gd": {}}, {"res://scripts/actions/meta_actions/ActionVariableCardsetModifier.gd": {"multiplied_values": ["draw_count"], "action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}]}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr"/>
@@ -2036,32 +2038,32 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>card_metronome</t>
+          <t>card_last_item</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>节拍器</t>
+          <t>最后一件</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>能力。每回合第一次打出攻击或技能时，其伤害和格挡提高 [value_bonus]。</t>
+          <t>造成 [damage] 点伤害。本场战斗每消耗过1张牌，额外造成 [damage_per_exhaust] 点伤害。</t>
         </is>
       </c>
       <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
         <v>2</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>color_green</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
       </c>
       <c r="H13" t="b">
         <v>0</v>
@@ -2070,7 +2072,7 @@
         <v>-1</v>
       </c>
       <c r="J13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
@@ -2086,17 +2088,19 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>external/sprites/cards/green/card_green.png</t>
+          <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>10</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="n">
-        <v>1</v>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
@@ -2109,22 +2113,18 @@
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>ActionApplyStatus</t>
+          <t>ActionVariableCombatStatsModifier</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr">
-        <is>
-          <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
-        </is>
-      </c>
+      <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="n">
         <v>1</v>
       </c>
       <c r="AL13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
@@ -2139,12 +2139,12 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>{"value_bonus": 2, "status_charge_amount": 1}</t>
+          <t>{"damage": 10, "damage_per_exhaust": 2, "number_of_attacks": 1}</t>
         </is>
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_metronome", "status_charge_amount": 1, "status_force_apply_new_effect": true, "status_custom_values": {"trigger_signal": "card_play_started", "max_triggers_per_turn": 1, "card_type_filter": [0, 1], "ignore_duplicate_plays": true, "action_data": [{"res://scripts/actions/meta_actions/ActionModifyCurrentCardPlayValues.gd": {"value_modifiers": {"damage": 2, "block": 2}, "operation": "add"}}]}}}]</t>
+          <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd": {"stat_enum": 14, "is_total_stat": true, "multiplied_values": ["damage"], "multiplied_values_bases": {"damage": 10}, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"damage": 2, "number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr"/>
@@ -2155,28 +2155,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>card_old_item_reuse</t>
+          <t>card_metronome</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>旧物回收</t>
+          <t>节拍器</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>放逐1张手牌。获得 [block] 点格挡，抽 [draw_count] 张牌。</t>
+          <t>能力。每回合第一次打出攻击或技能时，其伤害和格挡提高 [value_bonus]。</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>color_orange</t>
+          <t>color_green</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -2205,23 +2205,17 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>external/sprites/cards/orange/card_orange.png</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>keyword_exhaust,keyword_block</t>
-        </is>
-      </c>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="n">
-        <v>6</v>
-      </c>
-      <c r="T14" t="n">
-        <v>1</v>
-      </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
@@ -2234,21 +2228,25 @@
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>ActionPickCards</t>
+          <t>ActionApplyStatus</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
+        </is>
+      </c>
       <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="n">
         <v>1</v>
       </c>
-      <c r="AL14" t="inlineStr"/>
+      <c r="AL14" t="n">
+        <v>0</v>
+      </c>
       <c r="AM14" t="inlineStr"/>
-      <c r="AN14" t="n">
-        <v>3</v>
-      </c>
+      <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr"/>
@@ -2260,12 +2258,12 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>{"block": 6, "draw_count": 1, "min_card_amount": 1, "max_card_amount": 1}</t>
+          <t>{"value_bonus": 2, "status_charge_amount": 1}</t>
         </is>
       </c>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 0, "card_pick_text": "选择 {0} 张牌放逐。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionExhaustCards.gd": {}}, {"res://scripts/actions/ActionBlock.gd": {"target_override": 1, "time_delay": 0.5}}, {"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "actions_on_lethal": []}}]</t>
+          <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_metronome", "status_charge_amount": 1, "status_force_apply_new_effect": true, "status_custom_values": {"trigger_signal": "card_play_started", "max_triggers_per_turn": 1, "card_type_filter": [0, 1], "ignore_duplicate_plays": true, "action_data": [{"res://scripts/actions/meta_actions/ActionModifyCurrentCardPlayValues.gd": {"value_modifiers": {"damage": 2, "block": 2}, "operation": "add"}}]}}}]</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr"/>
@@ -2276,28 +2274,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>card_opening_strike</t>
+          <t>card_old_item_reuse</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>破绽打击</t>
+          <t>旧物回收</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>造成 [damage] 点伤害。如果目标正在攻击，施加 [status_charge_amount] 层易伤。</t>
+          <t>放逐1张手牌。获得 [block] 点格挡，抽 [draw_count] 张牌。</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>color_red</t>
+          <t>color_orange</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -2310,7 +2308,7 @@
         <v>-1</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
@@ -2326,30 +2324,28 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>external/sprites/cards/red/card_red.png</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="n">
-        <v>7</v>
-      </c>
-      <c r="R15" t="n">
-        <v>1</v>
-      </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="n">
-        <v>2</v>
-      </c>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>keyword_exhaust,keyword_block</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="n">
+        <v>6</v>
+      </c>
+      <c r="T15" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>status_effect_vulnerable</t>
-        </is>
-      </c>
+      <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
@@ -2357,12 +2353,10 @@
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>ActionAttackGenerator</t>
-        </is>
-      </c>
-      <c r="AG15" t="n">
-        <v>0</v>
-      </c>
+          <t>ActionPickCards</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
       <c r="AI15" t="inlineStr"/>
       <c r="AJ15" t="inlineStr"/>
@@ -2370,10 +2364,10 @@
         <v>1</v>
       </c>
       <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="n">
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="n">
         <v>3</v>
       </c>
-      <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
       <c r="AP15" t="inlineStr"/>
       <c r="AQ15" t="inlineStr"/>
@@ -2385,12 +2379,12 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>{"damage": 7, "number_of_attacks": 1, "status_charge_amount": 2, "status_effect_object_id": "status_effect_vulnerable"}</t>
+          <t>{"block": 6, "draw_count": 1, "min_card_amount": 1, "max_card_amount": 1}</t>
         </is>
       </c>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd": {}}], "passed_action_data": [{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"status_charge_amount": 2, "status_effect_object_id": "status_effect_vulnerable", "time_delay": 0.5, "actions_on_lethal": []}}], "failed_action_data": []}}]</t>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 0, "card_pick_text": "选择 {0} 张牌放逐。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionExhaustCards.gd": {}}, {"res://scripts/actions/ActionBlock.gd": {"target_override": 1, "time_delay": 0.5}}, {"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr"/>
@@ -2401,17 +2395,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>card_pursuit</t>
+          <t>card_opening_strike</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>追击</t>
+          <t>破绽打击</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>造成 [damage] 点伤害。若上一张牌是攻击，抽 [draw_count] 张牌。</t>
+          <t>造成 [damage] 点伤害。如果目标正在攻击，施加 [status_charge_amount] 层易伤。</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -2456,21 +2450,25 @@
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R16" t="n">
         <v>1</v>
       </c>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="n">
-        <v>1</v>
-      </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="n">
+        <v>2</v>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>status_effect_vulnerable</t>
+        </is>
+      </c>
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
@@ -2506,12 +2504,12 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>{"damage": 6, "number_of_attacks": 1, "draw_count": 1}</t>
+          <t>{"damage": 7, "number_of_attacks": 1, "status_charge_amount": 2, "status_effect_object_id": "status_effect_vulnerable"}</t>
         </is>
       </c>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "failed_action_data": []}}]</t>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd": {}}], "passed_action_data": [{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"status_charge_amount": 2, "status_effect_object_id": "status_effect_vulnerable", "time_delay": 0.5, "actions_on_lethal": []}}], "failed_action_data": []}}]</t>
         </is>
       </c>
       <c r="AX16" t="inlineStr"/>
@@ -2522,28 +2520,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>card_quick_search</t>
+          <t>card_pursuit</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>临时翻找</t>
+          <t>追击</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>从弃牌堆选择 [max_card_amount] 张牌加入手牌。本回合其费用变为0。</t>
+          <t>造成 [damage] 点伤害。若上一张牌是攻击，抽 [draw_count] 张牌。</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>color_blue</t>
+          <t>color_red</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -2556,7 +2554,7 @@
         <v>-1</v>
       </c>
       <c r="J17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
@@ -2572,14 +2570,20 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>external/sprites/cards/blue/card_blue.png</t>
+          <t>external/sprites/cards/red/card_red.png</t>
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>6</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
       <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="T17" t="n">
+        <v>1</v>
+      </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
@@ -2593,20 +2597,22 @@
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>ActionPickCards</t>
-        </is>
-      </c>
-      <c r="AG17" t="inlineStr"/>
+          <t>ActionAttackGenerator</t>
+        </is>
+      </c>
+      <c r="AG17" t="n">
+        <v>0</v>
+      </c>
       <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr"/>
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="n">
         <v>1</v>
       </c>
-      <c r="AL17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="n">
+        <v>3</v>
+      </c>
       <c r="AN17" t="inlineStr"/>
       <c r="AO17" t="inlineStr"/>
       <c r="AP17" t="inlineStr"/>
@@ -2619,12 +2625,12 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>{"min_card_amount": 1, "max_card_amount": 1}</t>
+          <t>{"damage": 6, "number_of_attacks": 1, "draw_count": 1}</t>
         </is>
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 4, "card_pick_text": "从弃牌堆选择 {0} 张牌。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionAddCardsToHand.gd": {}}, {"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd": {"card_energy_cost_until_turn": 0}}], "actions_on_lethal": []}}]</t>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "failed_action_data": []}}]</t>
         </is>
       </c>
       <c r="AX17" t="inlineStr"/>
@@ -2635,24 +2641,24 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>card_something_fell_out</t>
+          <t>card_quick_search</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>掉出来了</t>
+          <t>临时翻找</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>无法打出。被手动弃置时获得 [energy_amount] 点能量。</t>
+          <t>从弃牌堆选择 [max_card_amount] 张牌加入手牌。本回合其费用变为0。</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2688,11 +2694,7 @@
           <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>keyword_discard</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
@@ -2708,7 +2710,11 @@
       <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
       <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>ActionPickCards</t>
+        </is>
+      </c>
       <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="inlineStr"/>
       <c r="AI18" t="inlineStr"/>
@@ -2716,7 +2722,9 @@
       <c r="AK18" t="n">
         <v>1</v>
       </c>
-      <c r="AL18" t="inlineStr"/>
+      <c r="AL18" t="n">
+        <v>0</v>
+      </c>
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr"/>
@@ -2730,33 +2738,33 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>{"energy_amount": 2}</t>
-        </is>
-      </c>
-      <c r="AW18" t="inlineStr"/>
+          <t>{"min_card_amount": 1, "max_card_amount": 1}</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 4, "card_pick_text": "从弃牌堆选择 {0} 张牌。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionAddCardsToHand.gd": {}}, {"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd": {"card_energy_cost_until_turn": 0}}], "actions_on_lethal": []}}]</t>
+        </is>
+      </c>
       <c r="AX18" t="inlineStr"/>
-      <c r="AY18" t="inlineStr">
-        <is>
-          <t>[{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 2, "actions_on_lethal": []}}]</t>
-        </is>
-      </c>
+      <c r="AY18" t="inlineStr"/>
       <c r="AZ18" t="inlineStr"/>
       <c r="BA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>card_sports_drink</t>
+          <t>card_something_fell_out</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>运动饮料</t>
+          <t>掉出来了</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>抽到时获得 [energy_amount] 点能量。打出时抽 [draw_count] 张牌。放逐。</t>
+          <t>无法打出。被手动弃置时获得 [energy_amount] 点能量。</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -2767,7 +2775,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>color_orange</t>
+          <t>color_blue</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -2783,7 +2791,7 @@
         <v>0</v>
       </c>
       <c r="K19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" t="b">
         <v>0</v>
@@ -2796,20 +2804,18 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>external/sprites/cards/orange/card_orange.png</t>
+          <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>keyword_exhaust</t>
+          <t>keyword_discard</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
-      <c r="T19" t="n">
-        <v>1</v>
-      </c>
+      <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
@@ -2821,11 +2827,7 @@
       <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr">
-        <is>
-          <t>ActionDrawGenerator</t>
-        </is>
-      </c>
+      <c r="AF19" t="inlineStr"/>
       <c r="AG19" t="inlineStr"/>
       <c r="AH19" t="inlineStr"/>
       <c r="AI19" t="inlineStr"/>
@@ -2837,9 +2839,7 @@
       <c r="AM19" t="inlineStr"/>
       <c r="AN19" t="inlineStr"/>
       <c r="AO19" t="inlineStr"/>
-      <c r="AP19" t="n">
-        <v>1</v>
-      </c>
+      <c r="AP19" t="inlineStr"/>
       <c r="AQ19" t="inlineStr"/>
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr"/>
@@ -2849,44 +2849,40 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>{"energy_amount": 1, "draw_count": 1}</t>
-        </is>
-      </c>
-      <c r="AW19" t="inlineStr">
-        <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"actions_on_lethal": []}}]</t>
-        </is>
-      </c>
-      <c r="AX19" t="inlineStr">
-        <is>
-          <t>[{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 1, "actions_on_lethal": []}}]</t>
-        </is>
-      </c>
-      <c r="AY19" t="inlineStr"/>
+          <t>{"energy_amount": 2}</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 2, "actions_on_lethal": []}}]</t>
+        </is>
+      </c>
       <c r="AZ19" t="inlineStr"/>
       <c r="BA19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>card_sprint_start</t>
+          <t>card_sports_drink</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>冲刺起跑</t>
+          <t>运动饮料</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>抽到时，本回合费用变为0。造成 [damage] 点伤害。</t>
+          <t>抽到时获得 [energy_amount] 点能量。打出时抽 [draw_count] 张牌。放逐。</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -2894,7 +2890,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H20" t="b">
         <v>0</v>
@@ -2903,10 +2899,10 @@
         <v>-1</v>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" t="b">
         <v>0</v>
@@ -2922,15 +2918,17 @@
           <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="n">
-        <v>12</v>
-      </c>
-      <c r="R20" t="n">
-        <v>1</v>
-      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>keyword_exhaust</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
+      <c r="T20" t="n">
+        <v>1</v>
+      </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr"/>
@@ -2944,12 +2942,10 @@
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>ActionAttackGenerator</t>
-        </is>
-      </c>
-      <c r="AG20" t="n">
-        <v>0</v>
-      </c>
+          <t>ActionDrawGenerator</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr"/>
       <c r="AH20" t="inlineStr"/>
       <c r="AI20" t="inlineStr"/>
       <c r="AJ20" t="inlineStr"/>
@@ -2957,12 +2953,12 @@
         <v>1</v>
       </c>
       <c r="AL20" t="inlineStr"/>
-      <c r="AM20" t="n">
-        <v>4</v>
-      </c>
+      <c r="AM20" t="inlineStr"/>
       <c r="AN20" t="inlineStr"/>
       <c r="AO20" t="inlineStr"/>
-      <c r="AP20" t="inlineStr"/>
+      <c r="AP20" t="n">
+        <v>1</v>
+      </c>
       <c r="AQ20" t="inlineStr"/>
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="inlineStr"/>
@@ -2972,17 +2968,17 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>{"damage": 12, "number_of_attacks": 1}</t>
+          <t>{"energy_amount": 1, "draw_count": 1}</t>
         </is>
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}]</t>
+          <t>[{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"actions_on_lethal": []}}]</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd": {"pick_played_card": true, "card_energy_cost_until_turn": 0}}]</t>
+          <t>[{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 1, "actions_on_lethal": []}}]</t>
         </is>
       </c>
       <c r="AY20" t="inlineStr"/>
@@ -2992,21 +2988,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>card_travel_light</t>
+          <t>card_sprint_start</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>轻装上阵</t>
+          <t>冲刺起跑</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>能力。每回合第一次消耗牌时，获得 [energy_amount] 点能量。</t>
+          <t>抽到时，本回合费用变为0。造成 [damage] 点伤害。</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
@@ -3017,7 +3013,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" t="b">
         <v>0</v>
@@ -3026,7 +3022,7 @@
         <v>-1</v>
       </c>
       <c r="J21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="b">
         <v>0</v>
@@ -3046,13 +3042,15 @@
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="Q21" t="n">
+        <v>12</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
-      <c r="U21" t="n">
-        <v>1</v>
-      </c>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
@@ -3065,24 +3063,22 @@
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>ActionApplyStatus</t>
-        </is>
-      </c>
-      <c r="AG21" t="inlineStr"/>
-      <c r="AH21" t="inlineStr">
-        <is>
-          <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
-        </is>
-      </c>
+          <t>ActionAttackGenerator</t>
+        </is>
+      </c>
+      <c r="AG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="n">
         <v>1</v>
       </c>
-      <c r="AL21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="n">
+        <v>4</v>
+      </c>
       <c r="AN21" t="inlineStr"/>
       <c r="AO21" t="inlineStr"/>
       <c r="AP21" t="inlineStr"/>
@@ -3095,15 +3091,19 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>{"energy_amount": 1, "status_charge_amount": 1}</t>
+          <t>{"damage": 12, "number_of_attacks": 1}</t>
         </is>
       </c>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_travel_light", "status_charge_amount": 1, "status_force_apply_new_effect": true, "status_custom_values": {"trigger_signal": "card_exhausted", "max_triggers_per_turn": 1, "action_data": [{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 1}}]}}}]</t>
-        </is>
-      </c>
-      <c r="AX21" t="inlineStr"/>
+          <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}]</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd": {"pick_played_card": true, "card_energy_cost_until_turn": 0}}]</t>
+        </is>
+      </c>
       <c r="AY21" t="inlineStr"/>
       <c r="AZ21" t="inlineStr"/>
       <c r="BA21" t="inlineStr"/>
@@ -3111,28 +3111,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>card_tuning</t>
+          <t>card_travel_light</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>调音</t>
+          <t>轻装上阵</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>选择1张手牌。本场战斗中其伤害和格挡提高 [improve_amount]。放逐。</t>
+          <t>能力。每回合第一次消耗牌时，获得 [energy_amount] 点能量。</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>color_green</t>
+          <t>color_orange</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="K22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L22" t="b">
         <v>0</v>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>external/sprites/cards/green/card_green.png</t>
+          <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -3169,7 +3169,9 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="n">
+        <v>1</v>
+      </c>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
@@ -3182,17 +3184,23 @@
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>ActionPickCards</t>
+          <t>ActionApplyStatus</t>
         </is>
       </c>
       <c r="AG22" t="inlineStr"/>
-      <c r="AH22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
+        </is>
+      </c>
       <c r="AI22" t="inlineStr"/>
       <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="n">
         <v>1</v>
       </c>
-      <c r="AL22" t="inlineStr"/>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
       <c r="AM22" t="inlineStr"/>
       <c r="AN22" t="inlineStr"/>
       <c r="AO22" t="inlineStr"/>
@@ -3206,12 +3214,12 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>{"improve_amount": 2, "min_card_amount": 1, "max_card_amount": 1}</t>
+          <t>{"energy_amount": 1, "status_charge_amount": 1}</t>
         </is>
       </c>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 0, "card_pick_text": "选择 {0} 张牌调音。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd": {"improve_parent_card": false, "card_value_improvements": {"damage": 2, "block": 2}}}], "actions_on_lethal": []}}]</t>
+          <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_travel_light", "status_charge_amount": 1, "status_force_apply_new_effect": true, "status_custom_values": {"trigger_signal": "card_exhausted", "max_triggers_per_turn": 1, "action_data": [{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 1}}]}}}]</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr"/>
@@ -3222,28 +3230,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>card_warmup</t>
+          <t>card_tuning</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>赛前热身</t>
+          <t>调音</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>保留。获得 [block] 点格挡。每次被保留时，格挡提高 [improve_amount]。</t>
+          <t>选择1张手牌。本场战斗中其伤害和格挡提高 [improve_amount]。放逐。</t>
         </is>
       </c>
       <c r="D23" t="n">
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>color_orange</t>
+          <t>color_green</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -3259,32 +3267,26 @@
         <v>0</v>
       </c>
       <c r="K23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" t="b">
         <v>0</v>
       </c>
       <c r="M23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" t="b">
         <v>1</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>external/sprites/cards/orange/card_orange.png</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>keyword_block,keyword_retain</t>
-        </is>
-      </c>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
-      <c r="S23" t="n">
-        <v>6</v>
-      </c>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr"/>
@@ -3299,17 +3301,11 @@
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>ActionBlock</t>
-        </is>
-      </c>
-      <c r="AG23" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AH23" t="inlineStr">
-        <is>
-          <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
-        </is>
-      </c>
+          <t>ActionPickCards</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
       <c r="AI23" t="inlineStr"/>
       <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="n">
@@ -3317,9 +3313,7 @@
       </c>
       <c r="AL23" t="inlineStr"/>
       <c r="AM23" t="inlineStr"/>
-      <c r="AN23" t="n">
-        <v>2</v>
-      </c>
+      <c r="AN23" t="inlineStr"/>
       <c r="AO23" t="inlineStr"/>
       <c r="AP23" t="inlineStr"/>
       <c r="AQ23" t="inlineStr"/>
@@ -3331,22 +3325,147 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>{"block": 6, "improve_amount": 2}</t>
+          <t>{"improve_amount": 2, "min_card_amount": 1, "max_card_amount": 1}</t>
         </is>
       </c>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1, "actions_on_lethal": []}}]</t>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 0, "card_pick_text": "选择 {0} 张牌调音。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd": {"improve_parent_card": false, "card_value_improvements": {"damage": 2, "block": 2}}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr"/>
       <c r="AY23" t="inlineStr"/>
-      <c r="AZ23" t="inlineStr">
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>card_warmup</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>赛前热身</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>保留。获得 [block] 点格挡。每次被保留时，格挡提高 [improve_amount]。</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J24" t="b">
+        <v>0</v>
+      </c>
+      <c r="K24" t="b">
+        <v>0</v>
+      </c>
+      <c r="L24" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" t="b">
+        <v>1</v>
+      </c>
+      <c r="N24" t="b">
+        <v>1</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>keyword_block,keyword_retain</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="n">
+        <v>6</v>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>ActionBlock</t>
+        </is>
+      </c>
+      <c r="AG24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr"/>
+      <c r="AQ24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr"/>
+      <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>{"block": 6, "improve_amount": 2}</t>
+        </is>
+      </c>
+      <c r="AW24" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1, "actions_on_lethal": []}}]</t>
+        </is>
+      </c>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr">
         <is>
           <t>[{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd": {"pick_played_card": true, "improve_parent_card": false, "card_value_improvements": {"block": 2}}}]</t>
         </is>
       </c>
-      <c r="BA23" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add final card reference gap mechanics
</commit_message>
<xml_diff>
--- a/external/config/cards.xlsx
+++ b/external/config/cards.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA24"/>
+  <dimension ref="A1:BA28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -776,56 +776,6 @@
           <t>card_type: 0=攻击,1=技能,2=能力,3=状态,4=诅咒 | card_rarity: 0=基础,1=普通,2=稀有,3=罕见,4=生成</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -883,51 +833,26 @@
           <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
         <v>1</v>
       </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="n">
         <v>1</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
       </c>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr">
         <is>
           <t>ActionAddConsumable</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="n">
         <v>1</v>
       </c>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="n">
         <v>1</v>
       </c>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
       <c r="AU3" t="n">
         <v>0</v>
       </c>
@@ -941,10 +866,6 @@
           <t>[{"res://scripts/actions/player_actions/ActionAddConsumable.gd": {"random_consumable": 1, "fill_all_slots": 0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/ValidatorCombatStats.gd": {"stat_enum": 13, "is_total_stat": false, "operator": "&gt;", "comparison_value": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"actions_on_lethal": []}}], "failed_action_data": []}}]</t>
         </is>
       </c>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1002,26 +923,12 @@
           <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="n">
         <v>7</v>
       </c>
       <c r="R4" t="n">
         <v>1</v>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr">
         <is>
           <t>ActionAttackGenerator</t>
@@ -1030,23 +937,12 @@
       <c r="AG4" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="n">
         <v>1</v>
       </c>
-      <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="n">
         <v>3</v>
       </c>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
       <c r="AU4" t="n">
         <v>0</v>
       </c>
@@ -1060,10 +956,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/ValidatorCombatStats.gd": {"stat_enum": 14, "is_total_stat": false, "operator": "&gt;", "comparison_value": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"custom_key_names": {"damage": "bonus_damage"}, "number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}], "failed_action_data": []}}]</t>
         </is>
       </c>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1121,45 +1013,17 @@
           <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr">
         <is>
           <t>ActionPickCards</t>
         </is>
       </c>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="n">
         <v>1</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr"/>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
       <c r="AU5" t="n">
         <v>0</v>
       </c>
@@ -1173,10 +1037,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "random_selection": true, "card_pick_type": 4, "action_data": [{"res://scripts/actions/cardset_actions/ActionPlayCards.gd": {}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AX5" t="inlineStr"/>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1234,51 +1094,25 @@
           <t>external/sprites/cards/red/card_red.png</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="n">
         <v>3</v>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr">
         <is>
           <t>ActionApplyStatus</t>
         </is>
       </c>
-      <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr">
         <is>
           <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="n">
         <v>1</v>
       </c>
-      <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="n">
         <v>2</v>
       </c>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
       <c r="AU6" t="n">
         <v>0</v>
       </c>
@@ -1292,10 +1126,6 @@
           <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_combo_starter", "status_charge_amount": 1, "status_custom_values": {"card_type_filter": [0], "value_modifiers": {"damage": 3}, "consume_charge_on_trigger": true, "clear_on_player_turn_end": true, "ignore_duplicate_plays": true}}}]</t>
         </is>
       </c>
-      <c r="AX6" t="inlineStr"/>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1364,25 +1194,14 @@
       <c r="R7" t="n">
         <v>1</v>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
       <c r="U7" t="n">
         <v>4</v>
       </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr">
         <is>
           <t>status_effect_corrosion</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr">
         <is>
           <t>ActionAttackGenerator</t>
@@ -1391,25 +1210,15 @@
       <c r="AG7" t="n">
         <v>0</v>
       </c>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="n">
         <v>1</v>
       </c>
-      <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="n">
         <v>2</v>
       </c>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="n">
         <v>2</v>
       </c>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
       <c r="AU7" t="n">
         <v>0</v>
       </c>
@@ -1423,10 +1232,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"time_delay": 0.5, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd": {}}], "passed_action_data": [{"res://scripts/actions/enemy_actions/ActionCycleEnemyIntent.gd": {"time_delay": 0.0, "actions_on_lethal": []}}], "failed_action_data": []}}]</t>
         </is>
       </c>
-      <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1489,23 +1294,9 @@
           <t>keyword_block</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
         <v>7</v>
       </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr">
         <is>
           <t>ActionBlock</t>
@@ -1519,22 +1310,12 @@
           <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="n">
         <v>1</v>
       </c>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="n">
         <v>3</v>
       </c>
-      <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
       <c r="AU8" t="n">
         <v>0</v>
       </c>
@@ -1548,10 +1329,6 @@
           <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 1}}], "passed_action_data": [{"res://scripts/actions/ActionBlock.gd": {"custom_key_names": {"block": "bonus_block"}, "time_delay": 0.5, "target_override": 1}}], "failed_action_data": []}}]</t>
         </is>
       </c>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1620,42 +1397,17 @@
       <c r="R9" t="n">
         <v>1</v>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr">
         <is>
           <t>ActionTargetStatusValueModifier</t>
         </is>
       </c>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="n">
         <v>1</v>
       </c>
-      <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="n">
         <v>3</v>
       </c>
-      <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="inlineStr"/>
-      <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr"/>
-      <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr"/>
-      <c r="AT9" t="inlineStr"/>
       <c r="AU9" t="n">
         <v>0</v>
       </c>
@@ -1669,10 +1421,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionTargetStatusValueModifier.gd": {"status_effect_object_id": "status_effect_corrosion", "charge_key": "status_charges", "multiplier": 2, "value_key": "damage", "operation": "add", "default_value": 0, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
         </is>
       </c>
-      <c r="AX9" t="inlineStr"/>
-      <c r="AY9" t="inlineStr"/>
-      <c r="AZ9" t="inlineStr"/>
-      <c r="BA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1730,49 +1478,23 @@
           <t>external/sprites/cards/red/card_red.png</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
         <v>12</v>
       </c>
       <c r="R10" t="n">
         <v>1</v>
       </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr">
         <is>
           <t>ActionVariableCombatStatsModifier</t>
         </is>
       </c>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="n">
         <v>1</v>
       </c>
       <c r="AL10" t="n">
         <v>1</v>
       </c>
-      <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="inlineStr"/>
-      <c r="AO10" t="inlineStr"/>
-      <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr"/>
-      <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr"/>
-      <c r="AT10" t="inlineStr"/>
       <c r="AU10" t="n">
         <v>0</v>
       </c>
@@ -1786,10 +1508,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd": {"stat_enum": 11, "is_total_stat": false, "multiplied_values": ["damage"], "multiplied_values_bases": {"damage": 12}, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"damage": 3, "number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
         </is>
       </c>
-      <c r="AX10" t="inlineStr"/>
-      <c r="AY10" t="inlineStr"/>
-      <c r="AZ10" t="inlineStr"/>
-      <c r="BA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1852,25 +1570,12 @@
           <t>keyword_block</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
         <v>6</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr">
         <is>
           <t>ActionBlock</t>
@@ -1884,22 +1589,12 @@
           <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
         </is>
       </c>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="n">
         <v>1</v>
       </c>
-      <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="n">
         <v>3</v>
       </c>
-      <c r="AO11" t="inlineStr"/>
-      <c r="AP11" t="inlineStr"/>
-      <c r="AQ11" t="inlineStr"/>
-      <c r="AR11" t="inlineStr"/>
-      <c r="AS11" t="inlineStr"/>
-      <c r="AT11" t="inlineStr"/>
       <c r="AU11" t="n">
         <v>0</v>
       </c>
@@ -1913,10 +1608,6 @@
           <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/ValidatorCombatStats.gd": {"stat_enum": 11, "is_total_stat": false, "operator": "==", "comparison_value": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "failed_action_data": []}}]</t>
         </is>
       </c>
-      <c r="AX11" t="inlineStr"/>
-      <c r="AY11" t="inlineStr"/>
-      <c r="AZ11" t="inlineStr"/>
-      <c r="BA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1979,44 +1670,17 @@
           <t>keyword_discard</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
         <v>1</v>
       </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr">
         <is>
           <t>ActionPickCards</t>
         </is>
       </c>
-      <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="n">
         <v>1</v>
       </c>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="inlineStr"/>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr"/>
-      <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="inlineStr"/>
       <c r="AU12" t="n">
         <v>0</v>
       </c>
@@ -2030,10 +1694,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 0, "max_card_amount": 2, "card_pick_type": 0, "card_pick_text": "选择最多 {0} 张牌弃掉。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionDiscardCards.gd": {}}, {"res://scripts/actions/meta_actions/ActionVariableCardsetModifier.gd": {"multiplied_values": ["draw_count"], "action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}]}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AX12" t="inlineStr"/>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2091,49 +1751,23 @@
           <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
         <v>10</v>
       </c>
       <c r="R13" t="n">
         <v>1</v>
       </c>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr">
         <is>
           <t>ActionVariableCombatStatsModifier</t>
         </is>
       </c>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="n">
         <v>1</v>
       </c>
       <c r="AL13" t="n">
         <v>1</v>
       </c>
-      <c r="AM13" t="inlineStr"/>
-      <c r="AN13" t="inlineStr"/>
-      <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="inlineStr"/>
-      <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr"/>
-      <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="inlineStr"/>
       <c r="AU13" t="n">
         <v>0</v>
       </c>
@@ -2147,10 +1781,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionVariableCombatStatsModifier.gd": {"stat_enum": 14, "is_total_stat": true, "multiplied_values": ["damage"], "multiplied_values_bases": {"damage": 10}, "action_data": [{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"damage": 2, "number_of_attacks": 1, "time_delay": 0.0, "actions_on_lethal": []}}]}}]</t>
         </is>
       </c>
-      <c r="AX13" t="inlineStr"/>
-      <c r="AY13" t="inlineStr"/>
-      <c r="AZ13" t="inlineStr"/>
-      <c r="BA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2208,51 +1838,25 @@
           <t>external/sprites/cards/green/card_green.png</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
       <c r="U14" t="n">
         <v>1</v>
       </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr">
         <is>
           <t>ActionApplyStatus</t>
         </is>
       </c>
-      <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr">
         <is>
           <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
         </is>
       </c>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="n">
         <v>1</v>
       </c>
       <c r="AL14" t="n">
         <v>0</v>
       </c>
-      <c r="AM14" t="inlineStr"/>
-      <c r="AN14" t="inlineStr"/>
-      <c r="AO14" t="inlineStr"/>
-      <c r="AP14" t="inlineStr"/>
-      <c r="AQ14" t="inlineStr"/>
-      <c r="AR14" t="inlineStr"/>
-      <c r="AS14" t="inlineStr"/>
-      <c r="AT14" t="inlineStr"/>
       <c r="AU14" t="n">
         <v>0</v>
       </c>
@@ -2266,10 +1870,6 @@
           <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_metronome", "status_charge_amount": 1, "status_force_apply_new_effect": true, "status_custom_values": {"trigger_signal": "card_play_started", "max_triggers_per_turn": 1, "card_type_filter": [0, 1], "ignore_duplicate_plays": true, "action_data": [{"res://scripts/actions/meta_actions/ActionModifyCurrentCardPlayValues.gd": {"value_modifiers": {"damage": 2, "block": 2}, "operation": "add"}}]}}}]</t>
         </is>
       </c>
-      <c r="AX14" t="inlineStr"/>
-      <c r="AY14" t="inlineStr"/>
-      <c r="AZ14" t="inlineStr"/>
-      <c r="BA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2332,48 +1932,23 @@
           <t>keyword_exhaust,keyword_block</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
         <v>6</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
       </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
           <t>ActionPickCards</t>
         </is>
       </c>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="n">
         <v>1</v>
       </c>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="n">
         <v>3</v>
       </c>
-      <c r="AO15" t="inlineStr"/>
-      <c r="AP15" t="inlineStr"/>
-      <c r="AQ15" t="inlineStr"/>
-      <c r="AR15" t="inlineStr"/>
-      <c r="AS15" t="inlineStr"/>
-      <c r="AT15" t="inlineStr"/>
       <c r="AU15" t="n">
         <v>0</v>
       </c>
@@ -2387,10 +1962,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 0, "card_pick_text": "选择 {0} 张牌放逐。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionExhaustCards.gd": {}}, {"res://scripts/actions/ActionBlock.gd": {"target_override": 1, "time_delay": 0.5}}, {"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AX15" t="inlineStr"/>
-      <c r="AY15" t="inlineStr"/>
-      <c r="AZ15" t="inlineStr"/>
-      <c r="BA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2448,32 +2019,20 @@
           <t>external/sprites/cards/red/card_red.png</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
         <v>7</v>
       </c>
       <c r="R16" t="n">
         <v>1</v>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
       <c r="U16" t="n">
         <v>2</v>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr">
         <is>
           <t>status_effect_vulnerable</t>
         </is>
       </c>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr">
         <is>
           <t>ActionAttackGenerator</t>
@@ -2482,23 +2041,12 @@
       <c r="AG16" t="n">
         <v>0</v>
       </c>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="n">
         <v>1</v>
       </c>
-      <c r="AL16" t="inlineStr"/>
       <c r="AM16" t="n">
         <v>3</v>
       </c>
-      <c r="AN16" t="inlineStr"/>
-      <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr"/>
-      <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr"/>
-      <c r="AS16" t="inlineStr"/>
-      <c r="AT16" t="inlineStr"/>
       <c r="AU16" t="n">
         <v>0</v>
       </c>
@@ -2512,10 +2060,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorCardPlayEnemyAttacking.gd": {}}], "passed_action_data": [{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"status_charge_amount": 2, "status_effect_object_id": "status_effect_vulnerable", "time_delay": 0.5, "actions_on_lethal": []}}], "failed_action_data": []}}]</t>
         </is>
       </c>
-      <c r="AX16" t="inlineStr"/>
-      <c r="AY16" t="inlineStr"/>
-      <c r="AZ16" t="inlineStr"/>
-      <c r="BA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2573,28 +2117,15 @@
           <t>external/sprites/cards/red/card_red.png</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
       <c r="Q17" t="n">
         <v>6</v>
       </c>
       <c r="R17" t="n">
         <v>1</v>
       </c>
-      <c r="S17" t="inlineStr"/>
       <c r="T17" t="n">
         <v>1</v>
       </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
-      <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr">
         <is>
           <t>ActionAttackGenerator</t>
@@ -2603,23 +2134,12 @@
       <c r="AG17" t="n">
         <v>0</v>
       </c>
-      <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="n">
         <v>1</v>
       </c>
-      <c r="AL17" t="inlineStr"/>
       <c r="AM17" t="n">
         <v>3</v>
       </c>
-      <c r="AN17" t="inlineStr"/>
-      <c r="AO17" t="inlineStr"/>
-      <c r="AP17" t="inlineStr"/>
-      <c r="AQ17" t="inlineStr"/>
-      <c r="AR17" t="inlineStr"/>
-      <c r="AS17" t="inlineStr"/>
-      <c r="AT17" t="inlineStr"/>
       <c r="AU17" t="n">
         <v>0</v>
       </c>
@@ -2633,10 +2153,6 @@
           <t>[{"res://scripts/actions/meta_actions/ActionAttackGenerator.gd": {"time_delay": 0.0, "actions_on_lethal": []}}, {"res://scripts/actions/meta_actions/ActionValidator.gd": {"validator_data": [{"res://scripts/validators/card_plays/ValidatorPreviousCard.gd": {"card_type": 0}}], "passed_action_data": [{"res://scripts/actions/meta_actions/ActionDrawGenerator.gd": {"draw_count": 1}}], "failed_action_data": []}}]</t>
         </is>
       </c>
-      <c r="AX17" t="inlineStr"/>
-      <c r="AY17" t="inlineStr"/>
-      <c r="AZ17" t="inlineStr"/>
-      <c r="BA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2694,45 +2210,17 @@
           <t>external/sprites/cards/blue/card_blue.png</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr">
         <is>
           <t>ActionPickCards</t>
         </is>
       </c>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="n">
         <v>1</v>
       </c>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
-      <c r="AM18" t="inlineStr"/>
-      <c r="AN18" t="inlineStr"/>
-      <c r="AO18" t="inlineStr"/>
-      <c r="AP18" t="inlineStr"/>
-      <c r="AQ18" t="inlineStr"/>
-      <c r="AR18" t="inlineStr"/>
-      <c r="AS18" t="inlineStr"/>
-      <c r="AT18" t="inlineStr"/>
       <c r="AU18" t="n">
         <v>0</v>
       </c>
@@ -2746,10 +2234,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 4, "card_pick_text": "从弃牌堆选择 {0} 张牌。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionAddCardsToHand.gd": {}}, {"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd": {"card_energy_cost_until_turn": 0}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AX18" t="inlineStr"/>
-      <c r="AY18" t="inlineStr"/>
-      <c r="AZ18" t="inlineStr"/>
-      <c r="BA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2812,38 +2296,9 @@
           <t>keyword_discard</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="n">
         <v>1</v>
       </c>
-      <c r="AL19" t="inlineStr"/>
-      <c r="AM19" t="inlineStr"/>
-      <c r="AN19" t="inlineStr"/>
-      <c r="AO19" t="inlineStr"/>
-      <c r="AP19" t="inlineStr"/>
-      <c r="AQ19" t="inlineStr"/>
-      <c r="AR19" t="inlineStr"/>
-      <c r="AS19" t="inlineStr"/>
-      <c r="AT19" t="inlineStr"/>
       <c r="AU19" t="n">
         <v>0</v>
       </c>
@@ -2852,15 +2307,11 @@
           <t>{"energy_amount": 2}</t>
         </is>
       </c>
-      <c r="AW19" t="inlineStr"/>
-      <c r="AX19" t="inlineStr"/>
       <c r="AY19" t="inlineStr">
         <is>
           <t>[{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 2, "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AZ19" t="inlineStr"/>
-      <c r="BA19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2923,46 +2374,20 @@
           <t>keyword_exhaust</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
       <c r="T20" t="n">
         <v>1</v>
       </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr">
         <is>
           <t>ActionDrawGenerator</t>
         </is>
       </c>
-      <c r="AG20" t="inlineStr"/>
-      <c r="AH20" t="inlineStr"/>
-      <c r="AI20" t="inlineStr"/>
-      <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="n">
         <v>1</v>
       </c>
-      <c r="AL20" t="inlineStr"/>
-      <c r="AM20" t="inlineStr"/>
-      <c r="AN20" t="inlineStr"/>
-      <c r="AO20" t="inlineStr"/>
       <c r="AP20" t="n">
         <v>1</v>
       </c>
-      <c r="AQ20" t="inlineStr"/>
-      <c r="AR20" t="inlineStr"/>
-      <c r="AS20" t="inlineStr"/>
-      <c r="AT20" t="inlineStr"/>
       <c r="AU20" t="n">
         <v>0</v>
       </c>
@@ -2981,9 +2406,6 @@
           <t>[{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 1, "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AY20" t="inlineStr"/>
-      <c r="AZ20" t="inlineStr"/>
-      <c r="BA20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3041,26 +2463,12 @@
           <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr"/>
       <c r="Q21" t="n">
         <v>12</v>
       </c>
       <c r="R21" t="n">
         <v>1</v>
       </c>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
-      <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="inlineStr"/>
-      <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr">
         <is>
           <t>ActionAttackGenerator</t>
@@ -3069,23 +2477,12 @@
       <c r="AG21" t="n">
         <v>0</v>
       </c>
-      <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="n">
         <v>1</v>
       </c>
-      <c r="AL21" t="inlineStr"/>
       <c r="AM21" t="n">
         <v>4</v>
       </c>
-      <c r="AN21" t="inlineStr"/>
-      <c r="AO21" t="inlineStr"/>
-      <c r="AP21" t="inlineStr"/>
-      <c r="AQ21" t="inlineStr"/>
-      <c r="AR21" t="inlineStr"/>
-      <c r="AS21" t="inlineStr"/>
-      <c r="AT21" t="inlineStr"/>
       <c r="AU21" t="n">
         <v>0</v>
       </c>
@@ -3104,9 +2501,6 @@
           <t>[{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd": {"pick_played_card": true, "card_energy_cost_until_turn": 0}}]</t>
         </is>
       </c>
-      <c r="AY21" t="inlineStr"/>
-      <c r="AZ21" t="inlineStr"/>
-      <c r="BA21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3164,51 +2558,25 @@
           <t>external/sprites/cards/orange/card_orange.png</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
       <c r="U22" t="n">
         <v>1</v>
       </c>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr">
         <is>
           <t>ActionApplyStatus</t>
         </is>
       </c>
-      <c r="AG22" t="inlineStr"/>
       <c r="AH22" t="inlineStr">
         <is>
           <t>BaseAction.TARGET_OVERRIDES.PLAYER</t>
         </is>
       </c>
-      <c r="AI22" t="inlineStr"/>
-      <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="n">
         <v>1</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
-      <c r="AM22" t="inlineStr"/>
-      <c r="AN22" t="inlineStr"/>
-      <c r="AO22" t="inlineStr"/>
-      <c r="AP22" t="inlineStr"/>
-      <c r="AQ22" t="inlineStr"/>
-      <c r="AR22" t="inlineStr"/>
-      <c r="AS22" t="inlineStr"/>
-      <c r="AT22" t="inlineStr"/>
       <c r="AU22" t="n">
         <v>0</v>
       </c>
@@ -3222,10 +2590,6 @@
           <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_travel_light", "status_charge_amount": 1, "status_force_apply_new_effect": true, "status_custom_values": {"trigger_signal": "card_exhausted", "max_triggers_per_turn": 1, "action_data": [{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 1}}]}}}]</t>
         </is>
       </c>
-      <c r="AX22" t="inlineStr"/>
-      <c r="AY22" t="inlineStr"/>
-      <c r="AZ22" t="inlineStr"/>
-      <c r="BA22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3283,43 +2647,14 @@
           <t>external/sprites/cards/green/card_green.png</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr">
         <is>
           <t>ActionPickCards</t>
         </is>
       </c>
-      <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr"/>
-      <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="n">
         <v>1</v>
       </c>
-      <c r="AL23" t="inlineStr"/>
-      <c r="AM23" t="inlineStr"/>
-      <c r="AN23" t="inlineStr"/>
-      <c r="AO23" t="inlineStr"/>
-      <c r="AP23" t="inlineStr"/>
-      <c r="AQ23" t="inlineStr"/>
-      <c r="AR23" t="inlineStr"/>
-      <c r="AS23" t="inlineStr"/>
-      <c r="AT23" t="inlineStr"/>
       <c r="AU23" t="n">
         <v>0</v>
       </c>
@@ -3333,10 +2668,6 @@
           <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"min_card_amount": 1, "max_card_amount": 1, "min_cards_are_required_for_action": true, "card_pick_type": 0, "card_pick_text": "选择 {0} 张牌调音。已选择 {1} 张牌", "action_data": [{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd": {"improve_parent_card": false, "card_value_improvements": {"damage": 2, "block": 2}}}], "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AX23" t="inlineStr"/>
-      <c r="AY23" t="inlineStr"/>
-      <c r="AZ23" t="inlineStr"/>
-      <c r="BA23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3399,23 +2730,9 @@
           <t>keyword_block,keyword_retain</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
       <c r="S24" t="n">
         <v>6</v>
       </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr">
         <is>
           <t>ActionBlock</t>
@@ -3429,22 +2746,12 @@
           <t>BaseAction.TARGET_OVERRIDES.PARENT</t>
         </is>
       </c>
-      <c r="AI24" t="inlineStr"/>
-      <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="n">
         <v>1</v>
       </c>
-      <c r="AL24" t="inlineStr"/>
-      <c r="AM24" t="inlineStr"/>
       <c r="AN24" t="n">
         <v>2</v>
       </c>
-      <c r="AO24" t="inlineStr"/>
-      <c r="AP24" t="inlineStr"/>
-      <c r="AQ24" t="inlineStr"/>
-      <c r="AR24" t="inlineStr"/>
-      <c r="AS24" t="inlineStr"/>
-      <c r="AT24" t="inlineStr"/>
       <c r="AU24" t="n">
         <v>0</v>
       </c>
@@ -3458,14 +2765,475 @@
           <t>[{"res://scripts/actions/ActionBlock.gd": {"time_delay": 0.5, "target_override": 1, "actions_on_lethal": []}}]</t>
         </is>
       </c>
-      <c r="AX24" t="inlineStr"/>
-      <c r="AY24" t="inlineStr"/>
       <c r="AZ24" t="inlineStr">
         <is>
           <t>[{"res://scripts/actions/cardset_actions/ActionImproveCardValues.gd": {"pick_played_card": true, "improve_parent_card": false, "card_value_improvements": {"block": 2}}}]</t>
         </is>
       </c>
-      <c r="BA24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>card_chorus</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>副歌</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>能力。每回合第一次打出攻击或技能时，复制该牌一次。</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>color_green</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L25" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" t="b">
+        <v>1</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/green/card_green.png</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>1</v>
+      </c>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>ActionApplyStatus</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM25" t="inlineStr"/>
+      <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr"/>
+      <c r="AP25" t="inlineStr"/>
+      <c r="AQ25" t="inlineStr"/>
+      <c r="AR25" t="inlineStr"/>
+      <c r="AS25" t="inlineStr"/>
+      <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>{"status_charge_amount": 1}</t>
+        </is>
+      </c>
+      <c r="AW25" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_chorus", "status_charge_amount": 1, "status_force_apply_new_effect": true, "status_custom_values": {"trigger_signal": "card_play_started", "max_triggers_per_turn": 1, "card_type_filter": [0, 1], "ignore_duplicate_plays": true, "action_data": [{"res://scripts/actions/meta_actions/ActionDuplicateCurrentCardPlay.gd": {}}]}}}]</t>
+        </is>
+      </c>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr"/>
+      <c r="AZ25" t="inlineStr"/>
+      <c r="BA25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>card_bookmark_clip</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>夹好书签</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>选择1张手牌保留。下个玩家回合中，那张牌费用变为0。</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K26" t="b">
+        <v>0</v>
+      </c>
+      <c r="L26" t="b">
+        <v>0</v>
+      </c>
+      <c r="M26" t="b">
+        <v>0</v>
+      </c>
+      <c r="N26" t="b">
+        <v>1</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>keyword_retain</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>ActionPickCards</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" t="inlineStr"/>
+      <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="inlineStr"/>
+      <c r="AP26" t="inlineStr"/>
+      <c r="AQ26" t="inlineStr"/>
+      <c r="AR26" t="inlineStr"/>
+      <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="inlineStr"/>
+      <c r="AU26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"card_pick_type": 0, "min_card_amount": 1, "max_card_amount": 1, "card_pick_text": "选择1张牌夹好书签。{1}/{0}", "action_data": [{"res://scripts/actions/cardset_actions/ActionRetainCards.gd": {}}, {"res://scripts/actions/cardset_actions/ActionModifyCardTags.gd": {"add_tags": ["temporary_bookmark_clip_discount"]}}, {"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_bookmark_clip", "status_charge_amount": 1, "status_custom_values": {"trigger_signal": "player_turn_started", "activate_on_next_player_turn": true, "card_tag_filter": "temporary_bookmark_clip_discount", "remove_tag_on_trigger": false, "expire_on_player_turn_end": true, "action_data": [{"res://scripts/actions/cardset_actions/ActionChangeCardEnergies.gd": {"card_energy_cost_until_turn": 0}}]}}}]}}]</t>
+        </is>
+      </c>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
+      <c r="AZ26" t="inlineStr"/>
+      <c r="BA26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>card_pack_sorting</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>背包整理</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>选择1张手牌放到抽牌堆顶。下次抽到那张牌时，获得 [energy_amount] 点能量。</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J27" t="b">
+        <v>0</v>
+      </c>
+      <c r="K27" t="b">
+        <v>0</v>
+      </c>
+      <c r="L27" t="b">
+        <v>0</v>
+      </c>
+      <c r="M27" t="b">
+        <v>0</v>
+      </c>
+      <c r="N27" t="b">
+        <v>1</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>keyword_top_deck</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>ActionPickCards</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr"/>
+      <c r="AK27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL27" t="inlineStr"/>
+      <c r="AM27" t="inlineStr"/>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr"/>
+      <c r="AQ27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="inlineStr"/>
+      <c r="AU27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>{"energy_amount": 1}</t>
+        </is>
+      </c>
+      <c r="AW27" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"card_pick_type": 0, "min_card_amount": 1, "max_card_amount": 1, "card_pick_text": "选择1张牌放到抽牌堆顶。{1}/{0}", "action_data": [{"res://scripts/actions/cardset_actions/ActionModifyCardTags.gd": {"add_tags": ["temporary_pack_sorting_energy"]}}, {"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_pack_sorting", "status_charge_amount": 1, "status_custom_values": {"trigger_signal": "card_drawn", "card_tag_filter": "temporary_pack_sorting_energy", "remove_tag_on_trigger": true, "consume_charge_on_trigger": true, "action_data": [{"res://scripts/actions/ActionAddEnergy.gd": {"energy_amount": 1}}]}}}, {"res://scripts/actions/cardset_actions/ActionAddCardsToDraw.gd": {"card_destination": 4}}]}}]</t>
+        </is>
+      </c>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="inlineStr"/>
+      <c r="AZ27" t="inlineStr"/>
+      <c r="BA27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>card_ready_stance</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>准备姿态</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>保留所有攻击。下个玩家回合中，这些攻击造成额外 [damage] 点伤害。</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>color_orange</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J28" t="b">
+        <v>0</v>
+      </c>
+      <c r="K28" t="b">
+        <v>0</v>
+      </c>
+      <c r="L28" t="b">
+        <v>0</v>
+      </c>
+      <c r="M28" t="b">
+        <v>0</v>
+      </c>
+      <c r="N28" t="b">
+        <v>1</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>external/sprites/cards/orange/card_orange.png</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>keyword_retain</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>4</v>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>ActionPickCards</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr"/>
+      <c r="AQ28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV28" t="inlineStr">
+        <is>
+          <t>{"damage": 4}</t>
+        </is>
+      </c>
+      <c r="AW28" t="inlineStr">
+        <is>
+          <t>[{"res://scripts/actions/pick_card_actions/ActionPickCards.gd": {"card_pick_type": 0, "min_card_amount": 99, "max_card_amount": 99, "random_selection": true, "min_cards_are_required_for_action": false, "validator_data": [{"res://scripts/validators/card/ValidatorCardType.gd": {"card_types": [0]}}], "action_data": [{"res://scripts/actions/cardset_actions/ActionRetainCards.gd": {}}, {"res://scripts/actions/cardset_actions/ActionModifyCardTags.gd": {"add_tags": ["temporary_ready_stance_damage"]}}, {"res://scripts/actions/status_actions/ActionApplyStatus.gd": {"target_override": 2, "status_effect_object_id": "status_effect_ready_stance", "status_charge_amount": 1, "status_custom_values": {"trigger_signal": "card_play_started", "activate_on_next_player_turn": true, "card_tag_filter": "temporary_ready_stance_damage", "card_type_filter": [0], "ignore_duplicate_plays": true, "remove_tag_on_trigger": true, "expire_on_player_turn_end": true, "action_data": [{"res://scripts/actions/meta_actions/ActionModifyCurrentCardPlayValues.gd": {"value_modifiers": {"damage": 4}, "operation": "add"}}]}}}]}}]</t>
+        </is>
+      </c>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
+      <c r="AZ28" t="inlineStr"/>
+      <c r="BA28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
art: add individual red card illustrations
</commit_message>
<xml_diff>
--- a/external/config/cards.xlsx
+++ b/external/config/cards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="Rb42056beb47c459a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R2ab2d40956064374"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -982,7 +982,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/attack_lower_cost_on_discard_card.png</x:v>
       </x:c>
       <x:c r="P6"/>
       <x:c r="Q6" t="n">
@@ -1087,7 +1087,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O7" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/attack_with_conditional_block_card.png</x:v>
       </x:c>
       <x:c r="P7"/>
       <x:c r="Q7" t="n">
@@ -1194,7 +1194,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/attack_with_conditional_draw_card.png</x:v>
       </x:c>
       <x:c r="P8"/>
       <x:c r="Q8" t="n">
@@ -2453,7 +2453,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O20" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_banish_attack.png</x:v>
       </x:c>
       <x:c r="P20" t="str">
         <x:v>keyword_banish</x:v>
@@ -3885,7 +3885,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O34" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_discard_block.png</x:v>
       </x:c>
       <x:c r="P34" t="str">
         <x:v>keyword_block</x:v>
@@ -4398,7 +4398,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O39" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_draft_red_card.png</x:v>
       </x:c>
       <x:c r="P39"/>
       <x:c r="Q39"/>
@@ -4594,7 +4594,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O41" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_duplicate_attacks.png</x:v>
       </x:c>
       <x:c r="P41"/>
       <x:c r="Q41"/>
@@ -6002,7 +6002,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O55" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_law.png</x:v>
       </x:c>
       <x:c r="P55"/>
       <x:c r="Q55" t="n">
@@ -6309,7 +6309,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O58" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_opening_strike.png</x:v>
       </x:c>
       <x:c r="P58"/>
       <x:c r="Q58" t="n">
@@ -6715,7 +6715,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O62" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_play_random_from_hand.png</x:v>
       </x:c>
       <x:c r="P62"/>
       <x:c r="Q62"/>
@@ -6917,7 +6917,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O64" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_pursuit.png</x:v>
       </x:c>
       <x:c r="P64"/>
       <x:c r="Q64" t="n">
@@ -7222,7 +7222,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O67" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_requires_adjacency.png</x:v>
       </x:c>
       <x:c r="P67"/>
       <x:c r="Q67" t="n">
@@ -7517,7 +7517,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O70" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_right_click_transform_mode_a.png</x:v>
       </x:c>
       <x:c r="P70"/>
       <x:c r="Q70" t="n">
@@ -7619,7 +7619,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O71" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_right_click_transform_mode_b.png</x:v>
       </x:c>
       <x:c r="P71"/>
       <x:c r="Q71"/>
@@ -8508,7 +8508,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O80" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/card_vulnerable_enemies.png</x:v>
       </x:c>
       <x:c r="P80"/>
       <x:c r="Q80"/>
@@ -8825,7 +8825,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O83" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/cards_played_attack_card.png</x:v>
       </x:c>
       <x:c r="P83"/>
       <x:c r="Q83" t="n">
@@ -9130,7 +9130,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O86" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/ignore_damage_increase_attack_card.png</x:v>
       </x:c>
       <x:c r="P86"/>
       <x:c r="Q86" t="n">
@@ -9636,7 +9636,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O91" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/set_hand_energy_card.png</x:v>
       </x:c>
       <x:c r="P91"/>
       <x:c r="Q91"/>
@@ -9731,7 +9731,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O92" t="str">
-        <x:v>external/sprites/cards/red/card_red.png</x:v>
+        <x:v>external/sprites/cards/red/transform_hand_card.png</x:v>
       </x:c>
       <x:c r="P92"/>
       <x:c r="Q92"/>

</xml_diff>

<commit_message>
art: complete colored card illustrations
</commit_message>
<xml_diff>
--- a/external/config/cards.xlsx
+++ b/external/config/cards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R2ab2d40956064374"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R56af00f2d9fe41ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3188,7 +3188,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O27" t="str">
-        <x:v>external/sprites/cards/blue/card_blue.png</x:v>
+        <x:v>external/sprites/cards/blue/card_by_accident.png</x:v>
       </x:c>
       <x:c r="P27"/>
       <x:c r="Q27"/>
@@ -4087,7 +4087,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O36" t="str">
-        <x:v>external/sprites/cards/green/card_green.png</x:v>
+        <x:v>external/sprites/cards/green/card_distorted_note.png</x:v>
       </x:c>
       <x:c r="P36" t="str">
         <x:v>keyword_corrosion</x:v>
@@ -4806,7 +4806,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O43" t="str">
-        <x:v>external/sprites/cards/green/card_green.png</x:v>
+        <x:v>external/sprites/cards/green/card_echo_shield.png</x:v>
       </x:c>
       <x:c r="P43" t="str">
         <x:v>keyword_block</x:v>
@@ -5095,7 +5095,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O46" t="str">
-        <x:v>external/sprites/cards/green/card_green.png</x:v>
+        <x:v>external/sprites/cards/green/card_finale_burst.png</x:v>
       </x:c>
       <x:c r="P46" t="str">
         <x:v>keyword_corrosion</x:v>
@@ -5299,7 +5299,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O48" t="str">
-        <x:v>external/sprites/cards/green/card_green.png</x:v>
+        <x:v>external/sprites/cards/green/card_first_beat.png</x:v>
       </x:c>
       <x:c r="P48" t="str">
         <x:v>keyword_block</x:v>
@@ -5594,7 +5594,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O51" t="str">
-        <x:v>external/sprites/cards/blue/card_blue.png</x:v>
+        <x:v>external/sprites/cards/blue/card_hasty_sorting.png</x:v>
       </x:c>
       <x:c r="P51" t="str">
         <x:v>keyword_discard</x:v>
@@ -5901,7 +5901,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O54" t="str">
-        <x:v>external/sprites/cards/orange/card_orange.png</x:v>
+        <x:v>external/sprites/cards/orange/card_last_item.png</x:v>
       </x:c>
       <x:c r="P54"/>
       <x:c r="Q54" t="n">
@@ -6206,7 +6206,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O57" t="str">
-        <x:v>external/sprites/cards/orange/card_orange.png</x:v>
+        <x:v>external/sprites/cards/orange/card_old_item_reuse.png</x:v>
       </x:c>
       <x:c r="P57" t="str">
         <x:v>keyword_exhaust,keyword_block</x:v>
@@ -7022,7 +7022,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O65" t="str">
-        <x:v>external/sprites/cards/blue/card_blue.png</x:v>
+        <x:v>external/sprites/cards/blue/card_quick_search.png</x:v>
       </x:c>
       <x:c r="P65"/>
       <x:c r="Q65"/>
@@ -7819,7 +7819,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O73" t="str">
-        <x:v>external/sprites/cards/blue/card_blue.png</x:v>
+        <x:v>external/sprites/cards/blue/card_something_fell_out.png</x:v>
       </x:c>
       <x:c r="P73" t="str">
         <x:v>keyword_discard</x:v>
@@ -8011,7 +8011,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O75" t="str">
-        <x:v>external/sprites/cards/orange/card_orange.png</x:v>
+        <x:v>external/sprites/cards/orange/card_sports_drink.png</x:v>
       </x:c>
       <x:c r="P75" t="str">
         <x:v>keyword_exhaust</x:v>
@@ -8114,7 +8114,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O76" t="str">
-        <x:v>external/sprites/cards/orange/card_orange.png</x:v>
+        <x:v>external/sprites/cards/orange/card_sprint_start.png</x:v>
       </x:c>
       <x:c r="P76"/>
       <x:c r="Q76" t="n">
@@ -8219,7 +8219,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O77" t="str">
-        <x:v>external/sprites/cards/orange/card_orange.png</x:v>
+        <x:v>external/sprites/cards/orange/card_travel_light.png</x:v>
       </x:c>
       <x:c r="P77"/>
       <x:c r="Q77"/>
@@ -8320,7 +8320,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O78" t="str">
-        <x:v>external/sprites/cards/green/card_green.png</x:v>
+        <x:v>external/sprites/cards/green/card_tuning.png</x:v>
       </x:c>
       <x:c r="P78"/>
       <x:c r="Q78"/>
@@ -8613,7 +8613,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="O81" t="str">
-        <x:v>external/sprites/cards/orange/card_orange.png</x:v>
+        <x:v>external/sprites/cards/orange/card_warmup.png</x:v>
       </x:c>
       <x:c r="P81" t="str">
         <x:v>keyword_block,keyword_retain</x:v>

</xml_diff>

<commit_message>
art: add team card illustrations
</commit_message>
<xml_diff>
--- a/external/config/cards.xlsx
+++ b/external/config/cards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R56af00f2d9fe41ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="1" r:id="R1cba6e751bf64d31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -692,7 +692,9 @@
       <x:c r="N3" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O3"/>
+      <x:c r="O3" t="str">
+        <x:v>external/sprites/cards/white/add_health_card.png</x:v>
+      </x:c>
       <x:c r="P3"/>
       <x:c r="Q3"/>
       <x:c r="R3"/>
@@ -878,7 +880,9 @@
       <x:c r="N5" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O5"/>
+      <x:c r="O5" t="str">
+        <x:v>external/sprites/cards/purple/attack_increase_cost_on_damage_taken_card.png</x:v>
+      </x:c>
       <x:c r="P5"/>
       <x:c r="Q5" t="n">
         <x:v>7</x:v>
@@ -4910,7 +4914,9 @@
       <x:c r="N44" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O44"/>
+      <x:c r="O44" t="str">
+        <x:v>external/sprites/cards/purple/card_energy_on_discard.png</x:v>
+      </x:c>
       <x:c r="P44"/>
       <x:c r="Q44"/>
       <x:c r="R44"/>
@@ -7717,7 +7723,9 @@
       <x:c r="N72" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O72"/>
+      <x:c r="O72" t="str">
+        <x:v>external/sprites/cards/white/card_shove.png</x:v>
+      </x:c>
       <x:c r="P72"/>
       <x:c r="Q72" t="n">
         <x:v>4</x:v>
@@ -8929,7 +8937,9 @@
       <x:c r="N84" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O84"/>
+      <x:c r="O84" t="str">
+        <x:v>external/sprites/cards/white/custom_block_card.png</x:v>
+      </x:c>
       <x:c r="P84" t="str">
         <x:v>keyword_block</x:v>
       </x:c>
@@ -9028,7 +9038,9 @@
       <x:c r="N85" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O85"/>
+      <x:c r="O85" t="str">
+        <x:v>external/sprites/cards/white/end_turn_card.png</x:v>
+      </x:c>
       <x:c r="P85" t="str">
         <x:v>keyword_block</x:v>
       </x:c>
@@ -9234,7 +9246,9 @@
       <x:c r="N87" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O87"/>
+      <x:c r="O87" t="str">
+        <x:v>external/sprites/cards/purple/improving_retain_block_card.png</x:v>
+      </x:c>
       <x:c r="P87"/>
       <x:c r="Q87"/>
       <x:c r="R87"/>
@@ -9825,7 +9839,9 @@
       <x:c r="N93" s="2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O93"/>
+      <x:c r="O93" t="str">
+        <x:v>external/sprites/cards/purple/upgrade_entire_deck_card.png</x:v>
+      </x:c>
       <x:c r="P93"/>
       <x:c r="Q93"/>
       <x:c r="R93"/>

</xml_diff>